<commit_message>
Add audited 31 selected records; separate project guidance and prioritize 39-school coverage
</commit_message>
<xml_diff>
--- a/site/exports/pku-ic-microelectronics.xlsx
+++ b/site/exports/pku-ic-microelectronics.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R9c0b2d92d1a04b06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="Re8f144921bfd4eae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="R8a578f3f24d4473c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R1891e54c94414e98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="Rd3d774285c5e4f0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R6245712c83a54f4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="R77b0493074264f18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="R443a0927e3fc42dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="Rccb6cf4a9ef84806"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="R84b37080581d4016"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T7_0" displayName="T7_0" ref="A1:K11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T7_0" displayName="T7_0" ref="A1:K21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="校区"/>
@@ -158,7 +158,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T7_1" displayName="T7_1" ref="A1:S75" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T7_1" displayName="T7_1" ref="A1:S142" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="事件类型"/>
@@ -205,7 +205,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T7_3" displayName="T7_3" ref="A1:L22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T7_3" displayName="T7_3" ref="A1:L32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="标题"/>
@@ -225,7 +225,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T7_4" displayName="T7_4" ref="A1:G94" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T7_4" displayName="T7_4" ref="A1:G124" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="来源ID"/>
@@ -812,10 +812,340 @@
         <x:v>北京大学</x:v>
       </x:c>
     </x:row>
+    <x:row r="12" ht="64" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>黎明</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="str">
+        <x:v>校区未标注</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="str">
+        <x:v>集成电路学院·集成微纳电子系</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/lm/index.htm</x:v>
+      </x:c>
+      <x:c r="E12" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="str">
+        <x:v>各阶段导师未获直接确证；官网仅列成果总数，未由总数编造个人论文。</x:v>
+      </x:c>
+      <x:c r="G12" s="6" t="str">
+        <x:v>分批核实资料，不是完整名录</x:v>
+      </x:c>
+      <x:c r="H12" s="6" t="str">
+        <x:v>公开个人页（时效以核对日为准）</x:v>
+      </x:c>
+      <x:c r="I12" s="6" t="str"/>
+      <x:c r="J12" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="K12" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="64" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>刘力锋</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>校区未标注</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str">
+        <x:v>集成电路学院·集成微纳电子系</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/llf/index.htm</x:v>
+      </x:c>
+      <x:c r="E13" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="str">
+        <x:v>各阶段导师未获直接确证；官网仅列成果总数，未由总数编造个人论文。</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="str">
+        <x:v>分批核实资料，不是完整名录</x:v>
+      </x:c>
+      <x:c r="H13" s="6" t="str">
+        <x:v>公开个人页（时效以核对日为准）</x:v>
+      </x:c>
+      <x:c r="I13" s="6" t="str"/>
+      <x:c r="J13" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="K13" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="64" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>梁令</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="str">
+        <x:v>校区未标注</x:v>
+      </x:c>
+      <x:c r="C14" s="6" t="str">
+        <x:v>集成电路学院·集成微纳电子系</x:v>
+      </x:c>
+      <x:c r="D14" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/ll/index.htm</x:v>
+      </x:c>
+      <x:c r="E14" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F14" s="6" t="str">
+        <x:v>USC硕士原文笔误，授位待进一步确证。；UCSB论文索引可见委员会共同主席，但正文429未读取，候选不进入师承主图。；官网没有逐篇书目，本轮未扩充未经身份核定的合著论文。</x:v>
+      </x:c>
+      <x:c r="G14" s="6" t="str">
+        <x:v>分批核实资料，不是完整名录</x:v>
+      </x:c>
+      <x:c r="H14" s="6" t="str">
+        <x:v>公开个人页（时效以核对日为准）</x:v>
+      </x:c>
+      <x:c r="I14" s="6" t="str"/>
+      <x:c r="J14" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="K14" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="64" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>任黎明</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="str">
+        <x:v>校区未标注</x:v>
+      </x:c>
+      <x:c r="C15" s="6" t="str">
+        <x:v>集成电路学院·集成微纳电子系</x:v>
+      </x:c>
+      <x:c r="D15" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/rlm/index.htm</x:v>
+      </x:c>
+      <x:c r="E15" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F15" s="6" t="str">
+        <x:v>各阶段导师未获直接确证；官网仅列成果总数，未由总数编造个人论文。</x:v>
+      </x:c>
+      <x:c r="G15" s="6" t="str">
+        <x:v>分批核实资料，不是完整名录</x:v>
+      </x:c>
+      <x:c r="H15" s="6" t="str">
+        <x:v>公开个人页（时效以核对日为准）</x:v>
+      </x:c>
+      <x:c r="I15" s="6" t="str"/>
+      <x:c r="J15" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="K15" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="64" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>校区未标注</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="str">
+        <x:v>集成电路学院·集成微纳电子系</x:v>
+      </x:c>
+      <x:c r="D16" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="E16" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F16" s="6" t="str">
+        <x:v>本科/博士专业未披露；博士与博士后导师均未获直接确证，不由合著或实验室成员推师承。；研究员与助理教授两种原文并列保留；官网链接实验室当前读取失败，不补猜信息。</x:v>
+      </x:c>
+      <x:c r="G16" s="6" t="str">
+        <x:v>分批核实资料，不是完整名录</x:v>
+      </x:c>
+      <x:c r="H16" s="6" t="str">
+        <x:v>公开个人页（时效以核对日为准）</x:v>
+      </x:c>
+      <x:c r="I16" s="6" t="str"/>
+      <x:c r="J16" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="K16" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="64" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>孙雷</x:v>
+      </x:c>
+      <x:c r="B17" s="6" t="str">
+        <x:v>校区未标注</x:v>
+      </x:c>
+      <x:c r="C17" s="6" t="str">
+        <x:v>集成电路学院·集成微纳电子系</x:v>
+      </x:c>
+      <x:c r="D17" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="E17" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F17" s="6" t="str">
+        <x:v>导师未获已读取官方正文的直接确证；不从共同署名、实验室成员或招生导师称谓推定本人师承。；精选论文非全集；原始网页、论文PDF、联系人和学生信息不公开。</x:v>
+      </x:c>
+      <x:c r="G17" s="6" t="str">
+        <x:v>分批核实资料，不是完整名录</x:v>
+      </x:c>
+      <x:c r="H17" s="6" t="str">
+        <x:v>公开个人页（时效以核对日为准）</x:v>
+      </x:c>
+      <x:c r="I17" s="6" t="str"/>
+      <x:c r="J17" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="K17" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="64" customHeight="1">
+      <x:c r="A18" s="6" t="str">
+        <x:v>唐克超</x:v>
+      </x:c>
+      <x:c r="B18" s="6" t="str">
+        <x:v>校区未标注</x:v>
+      </x:c>
+      <x:c r="C18" s="6" t="str">
+        <x:v>集成电路学院·集成微纳电子系</x:v>
+      </x:c>
+      <x:c r="D18" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/tkc/index.htm</x:v>
+      </x:c>
+      <x:c r="E18" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F18" s="6" t="str">
+        <x:v>导师未获已读取官方正文的直接确证；不从共同署名、实验室成员或招生导师称谓推定本人师承。；精选论文非全集；原始网页、论文PDF、联系人和学生信息不公开。；博士导师Paul McIntyre候选来自官方新闻索引，当前正文无法取回，未入主图；博士后导师未获直接确证。；本人课题组页读取503；两篇RSC论文详情读取403后停止，未更换同页路由，未收入书目。</x:v>
+      </x:c>
+      <x:c r="G18" s="6" t="str">
+        <x:v>分批核实资料，不是完整名录</x:v>
+      </x:c>
+      <x:c r="H18" s="6" t="str">
+        <x:v>公开个人页（时效以核对日为准）</x:v>
+      </x:c>
+      <x:c r="I18" s="6" t="str"/>
+      <x:c r="J18" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="K18" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="64" customHeight="1">
+      <x:c r="A19" s="6" t="str">
+        <x:v>王宗巍</x:v>
+      </x:c>
+      <x:c r="B19" s="6" t="str">
+        <x:v>校区未标注</x:v>
+      </x:c>
+      <x:c r="C19" s="6" t="str">
+        <x:v>集成电路学院·集成微纳电子系</x:v>
+      </x:c>
+      <x:c r="D19" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wzw/index.htm</x:v>
+      </x:c>
+      <x:c r="E19" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F19" s="6" t="str">
+        <x:v>导师未获已读取官方正文的直接确证；不从共同署名、实验室成员或招生导师称谓推定本人师承。；精选论文非全集；原始网页、论文PDF、联系人和学生信息不公开。；国家自然科学基金委论文搜索索引称2018获博士，但原PDF已跳转到门户，未用未读正文填授位字段。；本人实验室网站返回客户端空壳，本轮未获得人物书目；官网论文总数不转成未核论文。</x:v>
+      </x:c>
+      <x:c r="G19" s="6" t="str">
+        <x:v>分批核实资料，不是完整名录</x:v>
+      </x:c>
+      <x:c r="H19" s="6" t="str">
+        <x:v>公开个人页（时效以核对日为准）</x:v>
+      </x:c>
+      <x:c r="I19" s="6" t="str"/>
+      <x:c r="J19" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="K19" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="64" customHeight="1">
+      <x:c r="A20" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B20" s="6" t="str">
+        <x:v>校区未标注</x:v>
+      </x:c>
+      <x:c r="C20" s="6" t="str">
+        <x:v>集成电路学院·集成微纳电子系</x:v>
+      </x:c>
+      <x:c r="D20" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="E20" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F20" s="6" t="str">
+        <x:v>导师未获已读取官方正文的直接确证；不从共同署名、实验室成员或招生导师称谓推定本人师承。；精选论文非全集；原始网页、论文PDF、联系人和学生信息不公开。</x:v>
+      </x:c>
+      <x:c r="G20" s="6" t="str">
+        <x:v>分批核实资料，不是完整名录</x:v>
+      </x:c>
+      <x:c r="H20" s="6" t="str">
+        <x:v>公开个人页（时效以核对日为准）</x:v>
+      </x:c>
+      <x:c r="I20" s="6" t="str"/>
+      <x:c r="J20" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="K20" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="64" customHeight="1">
+      <x:c r="A21" s="6" t="str">
+        <x:v>王茂俊</x:v>
+      </x:c>
+      <x:c r="B21" s="6" t="str">
+        <x:v>校区未标注</x:v>
+      </x:c>
+      <x:c r="C21" s="6" t="str">
+        <x:v>集成电路学院·集成微纳电子系</x:v>
+      </x:c>
+      <x:c r="D21" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wmj/index.htm</x:v>
+      </x:c>
+      <x:c r="E21" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F21" s="6" t="str">
+        <x:v>导师未获已读取官方正文的直接确证；不从共同署名、实验室成员或招生导师称谓推定本人师承。；精选论文非全集；原始网页、论文PDF、联系人和学生信息不公开。；2010-08至2011-07的任职未披露，不补连贯经历。；课题组主页503、本人学位论文机构库读取超时/503，本轮未由索引或合著补导师；官网只列成果总量，无逐篇书目。</x:v>
+      </x:c>
+      <x:c r="G21" s="6" t="str">
+        <x:v>分批核实资料，不是完整名录</x:v>
+      </x:c>
+      <x:c r="H21" s="6" t="str">
+        <x:v>公开个人页（时效以核对日为准）</x:v>
+      </x:c>
+      <x:c r="I21" s="6" t="str"/>
+      <x:c r="J21" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="K21" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96879bc6240e4280"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad74923965924711"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4248,10 +4578,3007 @@
         <x:v>北京大学</x:v>
       </x:c>
     </x:row>
+    <x:row r="76" ht="64" customHeight="1">
+      <x:c r="A76" s="6" t="str">
+        <x:v>黎明</x:v>
+      </x:c>
+      <x:c r="B76" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C76" s="6" t="str">
+        <x:v>学士</x:v>
+      </x:c>
+      <x:c r="D76" s="6" t="str">
+        <x:v>北京师范大学</x:v>
+      </x:c>
+      <x:c r="E76" s="6" t="str"/>
+      <x:c r="F76" s="6" t="str">
+        <x:v>1997</x:v>
+      </x:c>
+      <x:c r="G76" s="6" t="str">
+        <x:v>材料物理</x:v>
+      </x:c>
+      <x:c r="H76" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I76" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J76" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K76" s="6" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="L76" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M76" s="7" t="str"/>
+      <x:c r="N76" s="6" t="str"/>
+      <x:c r="O76" s="6" t="str"/>
+      <x:c r="P76" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q76" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/lm/index.htm</x:v>
+      </x:c>
+      <x:c r="R76" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S76" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="64" customHeight="1">
+      <x:c r="A77" s="6" t="str">
+        <x:v>黎明</x:v>
+      </x:c>
+      <x:c r="B77" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C77" s="6" t="str">
+        <x:v>硕士</x:v>
+      </x:c>
+      <x:c r="D77" s="6" t="str">
+        <x:v>北京师范大学</x:v>
+      </x:c>
+      <x:c r="E77" s="6" t="str"/>
+      <x:c r="F77" s="6" t="str">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G77" s="6" t="str">
+        <x:v>半导体科学与技术</x:v>
+      </x:c>
+      <x:c r="H77" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I77" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J77" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K77" s="6" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="L77" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M77" s="7" t="str"/>
+      <x:c r="N77" s="6" t="str"/>
+      <x:c r="O77" s="6" t="str"/>
+      <x:c r="P77" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q77" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/lm/index.htm</x:v>
+      </x:c>
+      <x:c r="R77" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S77" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="64" customHeight="1">
+      <x:c r="A78" s="6" t="str">
+        <x:v>黎明</x:v>
+      </x:c>
+      <x:c r="B78" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C78" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D78" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E78" s="6" t="str"/>
+      <x:c r="F78" s="6" t="str">
+        <x:v>2003</x:v>
+      </x:c>
+      <x:c r="G78" s="6" t="str">
+        <x:v>微电子与固体电子学</x:v>
+      </x:c>
+      <x:c r="H78" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I78" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J78" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K78" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L78" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M78" s="7" t="str"/>
+      <x:c r="N78" s="6" t="str"/>
+      <x:c r="O78" s="6" t="str">
+        <x:v>官网明确理学博士；各段起始年月未披露。</x:v>
+      </x:c>
+      <x:c r="P78" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q78" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/lm/index.htm</x:v>
+      </x:c>
+      <x:c r="R78" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S78" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="64" customHeight="1">
+      <x:c r="A79" s="6" t="str">
+        <x:v>黎明</x:v>
+      </x:c>
+      <x:c r="B79" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C79" s="6" t="str">
+        <x:v>长聘副教授，博导</x:v>
+      </x:c>
+      <x:c r="D79" s="6" t="str">
+        <x:v>北京大学集成电路学院</x:v>
+      </x:c>
+      <x:c r="E79" s="6" t="str"/>
+      <x:c r="F79" s="6" t="str"/>
+      <x:c r="G79" s="6" t="str"/>
+      <x:c r="H79" s="6" t="str"/>
+      <x:c r="I79" s="6" t="str"/>
+      <x:c r="J79" s="6" t="str"/>
+      <x:c r="K79" s="6" t="str"/>
+      <x:c r="L79" s="6" t="str"/>
+      <x:c r="M79" s="7" t="str"/>
+      <x:c r="N79" s="6" t="str"/>
+      <x:c r="O79" s="6" t="str">
+        <x:v>现行官方名录列示；不代表独立人事在岗核验，起始年月未知。</x:v>
+      </x:c>
+      <x:c r="P79" s="6" t="str"/>
+      <x:c r="Q79" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/lm/index.htm</x:v>
+      </x:c>
+      <x:c r="R79" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S79" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="64" customHeight="1">
+      <x:c r="A80" s="6" t="str">
+        <x:v>黎明</x:v>
+      </x:c>
+      <x:c r="B80" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C80" s="6" t="str">
+        <x:v>集成电路制造技术研发（职级未披露）</x:v>
+      </x:c>
+      <x:c r="D80" s="6" t="str">
+        <x:v>三星电子（韩国）半导体研究所</x:v>
+      </x:c>
+      <x:c r="E80" s="6" t="str">
+        <x:v>2003</x:v>
+      </x:c>
+      <x:c r="F80" s="6" t="str">
+        <x:v>2011</x:v>
+      </x:c>
+      <x:c r="G80" s="6" t="str"/>
+      <x:c r="H80" s="6" t="str"/>
+      <x:c r="I80" s="6" t="str"/>
+      <x:c r="J80" s="6" t="str"/>
+      <x:c r="K80" s="6" t="str"/>
+      <x:c r="L80" s="6" t="str"/>
+      <x:c r="M80" s="7" t="str"/>
+      <x:c r="N80" s="6" t="str"/>
+      <x:c r="O80" s="6" t="str"/>
+      <x:c r="P80" s="6" t="str"/>
+      <x:c r="Q80" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/lm/index.htm</x:v>
+      </x:c>
+      <x:c r="R80" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S80" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="64" customHeight="1">
+      <x:c r="A81" s="6" t="str">
+        <x:v>黎明</x:v>
+      </x:c>
+      <x:c r="B81" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C81" s="6" t="str">
+        <x:v>教学科研（具体职级起讫未披露）</x:v>
+      </x:c>
+      <x:c r="D81" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E81" s="6" t="str">
+        <x:v>2011</x:v>
+      </x:c>
+      <x:c r="F81" s="6" t="str"/>
+      <x:c r="G81" s="6" t="str"/>
+      <x:c r="H81" s="6" t="str"/>
+      <x:c r="I81" s="6" t="str"/>
+      <x:c r="J81" s="6" t="str"/>
+      <x:c r="K81" s="6" t="str"/>
+      <x:c r="L81" s="6" t="str"/>
+      <x:c r="M81" s="7" t="str"/>
+      <x:c r="N81" s="6" t="str"/>
+      <x:c r="O81" s="6" t="str"/>
+      <x:c r="P81" s="6" t="str"/>
+      <x:c r="Q81" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/lm/index.htm</x:v>
+      </x:c>
+      <x:c r="R81" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S81" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="64" customHeight="1">
+      <x:c r="A82" s="6" t="str">
+        <x:v>刘力锋</x:v>
+      </x:c>
+      <x:c r="B82" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C82" s="6" t="str">
+        <x:v>学士</x:v>
+      </x:c>
+      <x:c r="D82" s="6" t="str">
+        <x:v>河北工业大学</x:v>
+      </x:c>
+      <x:c r="E82" s="6" t="str"/>
+      <x:c r="F82" s="6" t="str">
+        <x:v>1999-07</x:v>
+      </x:c>
+      <x:c r="G82" s="6" t="str">
+        <x:v>电子工程</x:v>
+      </x:c>
+      <x:c r="H82" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I82" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J82" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K82" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L82" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M82" s="7" t="str"/>
+      <x:c r="N82" s="6" t="str"/>
+      <x:c r="O82" s="6" t="str"/>
+      <x:c r="P82" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q82" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/llf/index.htm</x:v>
+      </x:c>
+      <x:c r="R82" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S82" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="64" customHeight="1">
+      <x:c r="A83" s="6" t="str">
+        <x:v>刘力锋</x:v>
+      </x:c>
+      <x:c r="B83" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C83" s="6" t="str">
+        <x:v>硕士</x:v>
+      </x:c>
+      <x:c r="D83" s="6" t="str">
+        <x:v>河北工业大学</x:v>
+      </x:c>
+      <x:c r="E83" s="6" t="str"/>
+      <x:c r="F83" s="6" t="str">
+        <x:v>2002-03</x:v>
+      </x:c>
+      <x:c r="G83" s="6" t="str">
+        <x:v>微电子学与固体电子学</x:v>
+      </x:c>
+      <x:c r="H83" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I83" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J83" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K83" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L83" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M83" s="7" t="str"/>
+      <x:c r="N83" s="6" t="str"/>
+      <x:c r="O83" s="6" t="str"/>
+      <x:c r="P83" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q83" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/llf/index.htm</x:v>
+      </x:c>
+      <x:c r="R83" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S83" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="64" customHeight="1">
+      <x:c r="A84" s="6" t="str">
+        <x:v>刘力锋</x:v>
+      </x:c>
+      <x:c r="B84" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C84" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D84" s="6" t="str">
+        <x:v>中国科学院半导体研究所</x:v>
+      </x:c>
+      <x:c r="E84" s="6" t="str"/>
+      <x:c r="F84" s="6" t="str">
+        <x:v>2005-03</x:v>
+      </x:c>
+      <x:c r="G84" s="6" t="str">
+        <x:v>材料物理与化学</x:v>
+      </x:c>
+      <x:c r="H84" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I84" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J84" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K84" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L84" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M84" s="7" t="str"/>
+      <x:c r="N84" s="6" t="str"/>
+      <x:c r="O84" s="6" t="str"/>
+      <x:c r="P84" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q84" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/llf/index.htm</x:v>
+      </x:c>
+      <x:c r="R84" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S84" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="64" customHeight="1">
+      <x:c r="A85" s="6" t="str">
+        <x:v>刘力锋</x:v>
+      </x:c>
+      <x:c r="B85" s="6" t="str">
+        <x:v>postdoctoral_research</x:v>
+      </x:c>
+      <x:c r="C85" s="6" t="str"/>
+      <x:c r="D85" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E85" s="6" t="str">
+        <x:v>2005-04</x:v>
+      </x:c>
+      <x:c r="F85" s="6" t="str">
+        <x:v>2007-03</x:v>
+      </x:c>
+      <x:c r="G85" s="6" t="str"/>
+      <x:c r="H85" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I85" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J85" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K85" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L85" s="13" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M85" s="7" t="str"/>
+      <x:c r="N85" s="6" t="str"/>
+      <x:c r="O85" s="6" t="str">
+        <x:v>博士后科研经历，不是授予新学位。</x:v>
+      </x:c>
+      <x:c r="P85" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q85" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/llf/index.htm</x:v>
+      </x:c>
+      <x:c r="R85" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S85" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="64" customHeight="1">
+      <x:c r="A86" s="6" t="str">
+        <x:v>刘力锋</x:v>
+      </x:c>
+      <x:c r="B86" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C86" s="6" t="str">
+        <x:v>教授，博导</x:v>
+      </x:c>
+      <x:c r="D86" s="6" t="str">
+        <x:v>北京大学集成电路学院</x:v>
+      </x:c>
+      <x:c r="E86" s="6" t="str"/>
+      <x:c r="F86" s="6" t="str"/>
+      <x:c r="G86" s="6" t="str"/>
+      <x:c r="H86" s="6" t="str"/>
+      <x:c r="I86" s="6" t="str"/>
+      <x:c r="J86" s="6" t="str"/>
+      <x:c r="K86" s="6" t="str"/>
+      <x:c r="L86" s="6" t="str"/>
+      <x:c r="M86" s="7" t="str"/>
+      <x:c r="N86" s="6" t="str"/>
+      <x:c r="O86" s="6" t="str">
+        <x:v>现行官方名录列示；不代表独立人事在岗核验，起始年月未知。</x:v>
+      </x:c>
+      <x:c r="P86" s="6" t="str"/>
+      <x:c r="Q86" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/llf/index.htm</x:v>
+      </x:c>
+      <x:c r="R86" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S86" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="64" customHeight="1">
+      <x:c r="A87" s="6" t="str">
+        <x:v>刘力锋</x:v>
+      </x:c>
+      <x:c r="B87" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C87" s="6" t="str">
+        <x:v>博士后</x:v>
+      </x:c>
+      <x:c r="D87" s="6" t="str">
+        <x:v>北京大学信息科学技术学院微纳电子学系</x:v>
+      </x:c>
+      <x:c r="E87" s="6" t="str">
+        <x:v>2005-04</x:v>
+      </x:c>
+      <x:c r="F87" s="6" t="str">
+        <x:v>2007-03</x:v>
+      </x:c>
+      <x:c r="G87" s="6" t="str"/>
+      <x:c r="H87" s="6" t="str"/>
+      <x:c r="I87" s="6" t="str"/>
+      <x:c r="J87" s="6" t="str"/>
+      <x:c r="K87" s="6" t="str"/>
+      <x:c r="L87" s="6" t="str"/>
+      <x:c r="M87" s="7" t="str"/>
+      <x:c r="N87" s="6" t="str"/>
+      <x:c r="O87" s="6" t="str"/>
+      <x:c r="P87" s="6" t="str"/>
+      <x:c r="Q87" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/llf/index.htm</x:v>
+      </x:c>
+      <x:c r="R87" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S87" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="64" customHeight="1">
+      <x:c r="A88" s="6" t="str">
+        <x:v>刘力锋</x:v>
+      </x:c>
+      <x:c r="B88" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C88" s="6" t="str">
+        <x:v>留校工作（具体职级起讫未披露）</x:v>
+      </x:c>
+      <x:c r="D88" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E88" s="6" t="str">
+        <x:v>2007</x:v>
+      </x:c>
+      <x:c r="F88" s="6" t="str"/>
+      <x:c r="G88" s="6" t="str"/>
+      <x:c r="H88" s="6" t="str"/>
+      <x:c r="I88" s="6" t="str"/>
+      <x:c r="J88" s="6" t="str"/>
+      <x:c r="K88" s="6" t="str"/>
+      <x:c r="L88" s="6" t="str"/>
+      <x:c r="M88" s="7" t="str"/>
+      <x:c r="N88" s="6" t="str"/>
+      <x:c r="O88" s="6" t="str">
+        <x:v>原文博士后出站后留校；起年由出站年对应，未把出站月当精确聘任月。</x:v>
+      </x:c>
+      <x:c r="P88" s="6" t="str"/>
+      <x:c r="Q88" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/llf/index.htm</x:v>
+      </x:c>
+      <x:c r="R88" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S88" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="64" customHeight="1">
+      <x:c r="A89" s="6" t="str">
+        <x:v>梁令</x:v>
+      </x:c>
+      <x:c r="B89" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C89" s="6" t="str">
+        <x:v>学士</x:v>
+      </x:c>
+      <x:c r="D89" s="6" t="str">
+        <x:v>北京邮电大学</x:v>
+      </x:c>
+      <x:c r="E89" s="6" t="str">
+        <x:v>2011</x:v>
+      </x:c>
+      <x:c r="F89" s="6" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="G89" s="6" t="str">
+        <x:v>电子信息工程及管理</x:v>
+      </x:c>
+      <x:c r="H89" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I89" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J89" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K89" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L89" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M89" s="7" t="str"/>
+      <x:c r="N89" s="6" t="str"/>
+      <x:c r="O89" s="6" t="str"/>
+      <x:c r="P89" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q89" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/ll/index.htm</x:v>
+      </x:c>
+      <x:c r="R89" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S89" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="64" customHeight="1">
+      <x:c r="A90" s="6" t="str">
+        <x:v>梁令</x:v>
+      </x:c>
+      <x:c r="B90" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C90" s="6" t="str">
+        <x:v>硕士</x:v>
+      </x:c>
+      <x:c r="D90" s="6" t="str">
+        <x:v>南加州大学</x:v>
+      </x:c>
+      <x:c r="E90" s="6" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="F90" s="6" t="str">
+        <x:v>2017</x:v>
+      </x:c>
+      <x:c r="G90" s="6" t="str">
+        <x:v>电子工程</x:v>
+      </x:c>
+      <x:c r="H90" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="I90" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="J90" s="6" t="str">
+        <x:v>北美洲</x:v>
+      </x:c>
+      <x:c r="K90" s="6" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="L90" s="6" t="str"/>
+      <x:c r="M90" s="7" t="str"/>
+      <x:c r="N90" s="6" t="str"/>
+      <x:c r="O90" s="6" t="str">
+        <x:v>原文为“获得硕士专业”，疑似笔误；保留硕士经历但本轮不自动修文为明确授位。</x:v>
+      </x:c>
+      <x:c r="P90" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q90" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/ll/index.htm</x:v>
+      </x:c>
+      <x:c r="R90" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S90" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="64" customHeight="1">
+      <x:c r="A91" s="6" t="str">
+        <x:v>梁令</x:v>
+      </x:c>
+      <x:c r="B91" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C91" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D91" s="6" t="str">
+        <x:v>加州大学圣塔芭芭拉分校</x:v>
+      </x:c>
+      <x:c r="E91" s="6" t="str">
+        <x:v>2017</x:v>
+      </x:c>
+      <x:c r="F91" s="6" t="str">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="G91" s="6" t="str">
+        <x:v>电子计算机工程</x:v>
+      </x:c>
+      <x:c r="H91" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="I91" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="J91" s="6" t="str">
+        <x:v>北美洲</x:v>
+      </x:c>
+      <x:c r="K91" s="6" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="L91" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M91" s="7" t="str"/>
+      <x:c r="N91" s="6" t="str"/>
+      <x:c r="O91" s="6" t="str"/>
+      <x:c r="P91" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q91" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/ll/index.htm</x:v>
+      </x:c>
+      <x:c r="R91" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S91" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="64" customHeight="1">
+      <x:c r="A92" s="6" t="str">
+        <x:v>梁令</x:v>
+      </x:c>
+      <x:c r="B92" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C92" s="6" t="str">
+        <x:v>助理研究员</x:v>
+      </x:c>
+      <x:c r="D92" s="6" t="str">
+        <x:v>北京大学集成电路学院</x:v>
+      </x:c>
+      <x:c r="E92" s="6" t="str"/>
+      <x:c r="F92" s="6" t="str"/>
+      <x:c r="G92" s="6" t="str"/>
+      <x:c r="H92" s="6" t="str"/>
+      <x:c r="I92" s="6" t="str"/>
+      <x:c r="J92" s="6" t="str"/>
+      <x:c r="K92" s="6" t="str"/>
+      <x:c r="L92" s="6" t="str"/>
+      <x:c r="M92" s="7" t="str"/>
+      <x:c r="N92" s="6" t="str"/>
+      <x:c r="O92" s="6" t="str">
+        <x:v>现行官方名录列示；不代表独立人事在岗核验，起始年月未知。</x:v>
+      </x:c>
+      <x:c r="P92" s="6" t="str"/>
+      <x:c r="Q92" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/ll/index.htm</x:v>
+      </x:c>
+      <x:c r="R92" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S92" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="64" customHeight="1">
+      <x:c r="A93" s="6" t="str">
+        <x:v>梁令</x:v>
+      </x:c>
+      <x:c r="B93" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C93" s="6" t="str">
+        <x:v>隐私计算研究</x:v>
+      </x:c>
+      <x:c r="D93" s="6" t="str">
+        <x:v>阿里巴巴达摩院</x:v>
+      </x:c>
+      <x:c r="E93" s="6" t="str">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="F93" s="6" t="str">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G93" s="6" t="str"/>
+      <x:c r="H93" s="6" t="str"/>
+      <x:c r="I93" s="6" t="str"/>
+      <x:c r="J93" s="6" t="str"/>
+      <x:c r="K93" s="6" t="str"/>
+      <x:c r="L93" s="6" t="str"/>
+      <x:c r="M93" s="7" t="str"/>
+      <x:c r="N93" s="6" t="str"/>
+      <x:c r="O93" s="6" t="str"/>
+      <x:c r="P93" s="6" t="str"/>
+      <x:c r="Q93" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/ll/index.htm</x:v>
+      </x:c>
+      <x:c r="R93" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S93" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="64" customHeight="1">
+      <x:c r="A94" s="6" t="str">
+        <x:v>梁令</x:v>
+      </x:c>
+      <x:c r="B94" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C94" s="6" t="str">
+        <x:v>助理研究员</x:v>
+      </x:c>
+      <x:c r="D94" s="6" t="str">
+        <x:v>北京大学集成电路学院</x:v>
+      </x:c>
+      <x:c r="E94" s="6" t="str">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="F94" s="6" t="str"/>
+      <x:c r="G94" s="6" t="str"/>
+      <x:c r="H94" s="6" t="str"/>
+      <x:c r="I94" s="6" t="str"/>
+      <x:c r="J94" s="6" t="str"/>
+      <x:c r="K94" s="6" t="str"/>
+      <x:c r="L94" s="6" t="str"/>
+      <x:c r="M94" s="7" t="str"/>
+      <x:c r="N94" s="6" t="str"/>
+      <x:c r="O94" s="6" t="str"/>
+      <x:c r="P94" s="6" t="str"/>
+      <x:c r="Q94" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/ll/index.htm</x:v>
+      </x:c>
+      <x:c r="R94" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S94" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="64" customHeight="1">
+      <x:c r="A95" s="6" t="str">
+        <x:v>任黎明</x:v>
+      </x:c>
+      <x:c r="B95" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C95" s="6" t="str">
+        <x:v>学士</x:v>
+      </x:c>
+      <x:c r="D95" s="6" t="str">
+        <x:v>山东大学</x:v>
+      </x:c>
+      <x:c r="E95" s="6" t="str">
+        <x:v>1990-09</x:v>
+      </x:c>
+      <x:c r="F95" s="6" t="str">
+        <x:v>1994-07</x:v>
+      </x:c>
+      <x:c r="G95" s="6" t="str">
+        <x:v>半导体物理与器件</x:v>
+      </x:c>
+      <x:c r="H95" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I95" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J95" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K95" s="6" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="L95" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M95" s="7" t="str"/>
+      <x:c r="N95" s="6" t="str"/>
+      <x:c r="O95" s="6" t="str"/>
+      <x:c r="P95" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q95" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/rlm/index.htm</x:v>
+      </x:c>
+      <x:c r="R95" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S95" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="64" customHeight="1">
+      <x:c r="A96" s="6" t="str">
+        <x:v>任黎明</x:v>
+      </x:c>
+      <x:c r="B96" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C96" s="6" t="str">
+        <x:v>硕士</x:v>
+      </x:c>
+      <x:c r="D96" s="6" t="str">
+        <x:v>山东大学</x:v>
+      </x:c>
+      <x:c r="E96" s="6" t="str">
+        <x:v>1996-09</x:v>
+      </x:c>
+      <x:c r="F96" s="6" t="str">
+        <x:v>1999-07</x:v>
+      </x:c>
+      <x:c r="G96" s="6" t="str">
+        <x:v>电力系统及其自动化</x:v>
+      </x:c>
+      <x:c r="H96" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I96" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J96" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K96" s="6" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="L96" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M96" s="7" t="str"/>
+      <x:c r="N96" s="6" t="str"/>
+      <x:c r="O96" s="6" t="str"/>
+      <x:c r="P96" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q96" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/rlm/index.htm</x:v>
+      </x:c>
+      <x:c r="R96" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S96" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="64" customHeight="1">
+      <x:c r="A97" s="6" t="str">
+        <x:v>任黎明</x:v>
+      </x:c>
+      <x:c r="B97" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C97" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D97" s="6" t="str">
+        <x:v>中国科学院微电子研究所</x:v>
+      </x:c>
+      <x:c r="E97" s="6" t="str">
+        <x:v>1999-09</x:v>
+      </x:c>
+      <x:c r="F97" s="6" t="str">
+        <x:v>2002-07</x:v>
+      </x:c>
+      <x:c r="G97" s="6" t="str">
+        <x:v>微电子学与固体电子学</x:v>
+      </x:c>
+      <x:c r="H97" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I97" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J97" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K97" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L97" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M97" s="7" t="str"/>
+      <x:c r="N97" s="6" t="str"/>
+      <x:c r="O97" s="6" t="str"/>
+      <x:c r="P97" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q97" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/rlm/index.htm</x:v>
+      </x:c>
+      <x:c r="R97" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S97" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="64" customHeight="1">
+      <x:c r="A98" s="6" t="str">
+        <x:v>任黎明</x:v>
+      </x:c>
+      <x:c r="B98" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C98" s="6" t="str">
+        <x:v>讲师</x:v>
+      </x:c>
+      <x:c r="D98" s="6" t="str">
+        <x:v>北京大学集成电路学院</x:v>
+      </x:c>
+      <x:c r="E98" s="6" t="str"/>
+      <x:c r="F98" s="6" t="str"/>
+      <x:c r="G98" s="6" t="str"/>
+      <x:c r="H98" s="6" t="str"/>
+      <x:c r="I98" s="6" t="str"/>
+      <x:c r="J98" s="6" t="str"/>
+      <x:c r="K98" s="6" t="str"/>
+      <x:c r="L98" s="6" t="str"/>
+      <x:c r="M98" s="7" t="str"/>
+      <x:c r="N98" s="6" t="str"/>
+      <x:c r="O98" s="6" t="str">
+        <x:v>现行官方名录列示；不代表独立人事在岗核验，起始年月未知。</x:v>
+      </x:c>
+      <x:c r="P98" s="6" t="str"/>
+      <x:c r="Q98" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/rlm/index.htm</x:v>
+      </x:c>
+      <x:c r="R98" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S98" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="64" customHeight="1">
+      <x:c r="A99" s="6" t="str">
+        <x:v>任黎明</x:v>
+      </x:c>
+      <x:c r="B99" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C99" s="6" t="str">
+        <x:v>任教</x:v>
+      </x:c>
+      <x:c r="D99" s="6" t="str">
+        <x:v>山东省烟台市化工管理干部培训学校</x:v>
+      </x:c>
+      <x:c r="E99" s="6" t="str">
+        <x:v>1994-07</x:v>
+      </x:c>
+      <x:c r="F99" s="6" t="str">
+        <x:v>1996-08</x:v>
+      </x:c>
+      <x:c r="G99" s="6" t="str"/>
+      <x:c r="H99" s="6" t="str"/>
+      <x:c r="I99" s="6" t="str"/>
+      <x:c r="J99" s="6" t="str"/>
+      <x:c r="K99" s="6" t="str"/>
+      <x:c r="L99" s="6" t="str"/>
+      <x:c r="M99" s="7" t="str"/>
+      <x:c r="N99" s="6" t="str"/>
+      <x:c r="O99" s="6" t="str"/>
+      <x:c r="P99" s="6" t="str"/>
+      <x:c r="Q99" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/rlm/index.htm</x:v>
+      </x:c>
+      <x:c r="R99" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S99" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="64" customHeight="1">
+      <x:c r="A100" s="6" t="str">
+        <x:v>任黎明</x:v>
+      </x:c>
+      <x:c r="B100" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C100" s="6" t="str">
+        <x:v>教学科研</x:v>
+      </x:c>
+      <x:c r="D100" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E100" s="6" t="str">
+        <x:v>2002-07</x:v>
+      </x:c>
+      <x:c r="F100" s="6" t="str"/>
+      <x:c r="G100" s="6" t="str"/>
+      <x:c r="H100" s="6" t="str"/>
+      <x:c r="I100" s="6" t="str"/>
+      <x:c r="J100" s="6" t="str"/>
+      <x:c r="K100" s="6" t="str"/>
+      <x:c r="L100" s="6" t="str"/>
+      <x:c r="M100" s="7" t="str"/>
+      <x:c r="N100" s="6" t="str"/>
+      <x:c r="O100" s="6" t="str"/>
+      <x:c r="P100" s="6" t="str"/>
+      <x:c r="Q100" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/rlm/index.htm</x:v>
+      </x:c>
+      <x:c r="R100" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S100" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="64" customHeight="1">
+      <x:c r="A101" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B101" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C101" s="6" t="str">
+        <x:v>学士</x:v>
+      </x:c>
+      <x:c r="D101" s="6" t="str">
+        <x:v>南开大学</x:v>
+      </x:c>
+      <x:c r="E101" s="6" t="str">
+        <x:v>2007</x:v>
+      </x:c>
+      <x:c r="F101" s="6" t="str">
+        <x:v>2011</x:v>
+      </x:c>
+      <x:c r="G101" s="6" t="str"/>
+      <x:c r="H101" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I101" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J101" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K101" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L101" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M101" s="7" t="str"/>
+      <x:c r="N101" s="6" t="str"/>
+      <x:c r="O101" s="6" t="str"/>
+      <x:c r="P101" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q101" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="R101" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S101" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="64" customHeight="1">
+      <x:c r="A102" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B102" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C102" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D102" s="6" t="str">
+        <x:v>清华大学</x:v>
+      </x:c>
+      <x:c r="E102" s="6" t="str">
+        <x:v>2011</x:v>
+      </x:c>
+      <x:c r="F102" s="6" t="str">
+        <x:v>2016</x:v>
+      </x:c>
+      <x:c r="G102" s="6" t="str"/>
+      <x:c r="H102" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I102" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J102" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K102" s="6" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="L102" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M102" s="7" t="str"/>
+      <x:c r="N102" s="6" t="str"/>
+      <x:c r="O102" s="6" t="str"/>
+      <x:c r="P102" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q102" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="R102" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S102" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="64" customHeight="1">
+      <x:c r="A103" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B103" s="6" t="str">
+        <x:v>postdoctoral_research</x:v>
+      </x:c>
+      <x:c r="C103" s="6" t="str"/>
+      <x:c r="D103" s="6" t="str">
+        <x:v>米兰理工大学</x:v>
+      </x:c>
+      <x:c r="E103" s="6" t="str">
+        <x:v>2016</x:v>
+      </x:c>
+      <x:c r="F103" s="6" t="str">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="G103" s="6" t="str"/>
+      <x:c r="H103" s="6" t="str">
+        <x:v>意大利</x:v>
+      </x:c>
+      <x:c r="I103" s="6" t="str">
+        <x:v>意大利</x:v>
+      </x:c>
+      <x:c r="J103" s="6" t="str">
+        <x:v>欧洲</x:v>
+      </x:c>
+      <x:c r="K103" s="6" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="L103" s="13" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M103" s="7" t="str"/>
+      <x:c r="N103" s="6" t="str"/>
+      <x:c r="O103" s="6" t="str"/>
+      <x:c r="P103" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q103" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="R103" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S103" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="64" customHeight="1">
+      <x:c r="A104" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B104" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C104" s="6" t="str">
+        <x:v>助理教授，博导</x:v>
+      </x:c>
+      <x:c r="D104" s="6" t="str">
+        <x:v>北京大学集成电路学院</x:v>
+      </x:c>
+      <x:c r="E104" s="6" t="str"/>
+      <x:c r="F104" s="6" t="str"/>
+      <x:c r="G104" s="6" t="str"/>
+      <x:c r="H104" s="6" t="str"/>
+      <x:c r="I104" s="6" t="str"/>
+      <x:c r="J104" s="6" t="str"/>
+      <x:c r="K104" s="6" t="str"/>
+      <x:c r="L104" s="6" t="str"/>
+      <x:c r="M104" s="7" t="str"/>
+      <x:c r="N104" s="6" t="str"/>
+      <x:c r="O104" s="6" t="str">
+        <x:v>现行官方名录列示；不代表独立人事在岗核验，起始年月未知。</x:v>
+      </x:c>
+      <x:c r="P104" s="6" t="str"/>
+      <x:c r="Q104" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="R104" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S104" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="64" customHeight="1">
+      <x:c r="A105" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B105" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C105" s="6" t="str">
+        <x:v>博士后</x:v>
+      </x:c>
+      <x:c r="D105" s="6" t="str">
+        <x:v>米兰理工大学</x:v>
+      </x:c>
+      <x:c r="E105" s="6" t="str">
+        <x:v>2016</x:v>
+      </x:c>
+      <x:c r="F105" s="6" t="str">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="G105" s="6" t="str"/>
+      <x:c r="H105" s="6" t="str"/>
+      <x:c r="I105" s="6" t="str"/>
+      <x:c r="J105" s="6" t="str"/>
+      <x:c r="K105" s="6" t="str"/>
+      <x:c r="L105" s="6" t="str"/>
+      <x:c r="M105" s="7" t="str"/>
+      <x:c r="N105" s="6" t="str"/>
+      <x:c r="O105" s="6" t="str"/>
+      <x:c r="P105" s="6" t="str"/>
+      <x:c r="Q105" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="R105" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S105" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="64" customHeight="1">
+      <x:c r="A106" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B106" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C106" s="6" t="str">
+        <x:v>研究员、北大博雅青年学者</x:v>
+      </x:c>
+      <x:c r="D106" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E106" s="6" t="str">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="F106" s="6" t="str"/>
+      <x:c r="G106" s="6" t="str"/>
+      <x:c r="H106" s="6" t="str"/>
+      <x:c r="I106" s="6" t="str"/>
+      <x:c r="J106" s="6" t="str"/>
+      <x:c r="K106" s="6" t="str"/>
+      <x:c r="L106" s="6" t="str"/>
+      <x:c r="M106" s="7" t="str"/>
+      <x:c r="N106" s="6" t="str"/>
+      <x:c r="O106" s="6" t="str">
+        <x:v>本人页头部为助理教授、正文为研究员，保留岗位/职称不同口径，不推断晋升日期。</x:v>
+      </x:c>
+      <x:c r="P106" s="6" t="str"/>
+      <x:c r="Q106" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="R106" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S106" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="64" customHeight="1">
+      <x:c r="A107" s="6" t="str">
+        <x:v>孙雷</x:v>
+      </x:c>
+      <x:c r="B107" s="6" t="str">
+        <x:v>degree_study</x:v>
+      </x:c>
+      <x:c r="C107" s="6" t="str">
+        <x:v>本科</x:v>
+      </x:c>
+      <x:c r="D107" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E107" s="6" t="str"/>
+      <x:c r="F107" s="6" t="str">
+        <x:v>1997</x:v>
+      </x:c>
+      <x:c r="G107" s="6" t="str"/>
+      <x:c r="H107" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I107" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J107" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K107" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L107" s="6" t="str"/>
+      <x:c r="M107" s="7" t="str"/>
+      <x:c r="N107" s="6" t="str"/>
+      <x:c r="O107" s="6" t="str">
+        <x:v>原文为本科/硕士/博士毕业，未另见明确获授学位表述；起始年月和专业未披露。</x:v>
+      </x:c>
+      <x:c r="P107" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q107" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="R107" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S107" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="64" customHeight="1">
+      <x:c r="A108" s="6" t="str">
+        <x:v>孙雷</x:v>
+      </x:c>
+      <x:c r="B108" s="6" t="str">
+        <x:v>degree_study</x:v>
+      </x:c>
+      <x:c r="C108" s="6" t="str">
+        <x:v>硕士</x:v>
+      </x:c>
+      <x:c r="D108" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E108" s="6" t="str"/>
+      <x:c r="F108" s="6" t="str">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="G108" s="6" t="str"/>
+      <x:c r="H108" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I108" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J108" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K108" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L108" s="6" t="str"/>
+      <x:c r="M108" s="7" t="str"/>
+      <x:c r="N108" s="6" t="str"/>
+      <x:c r="O108" s="6" t="str">
+        <x:v>原文为本科/硕士/博士毕业，未另见明确获授学位表述；起始年月和专业未披露。</x:v>
+      </x:c>
+      <x:c r="P108" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q108" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="R108" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S108" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="64" customHeight="1">
+      <x:c r="A109" s="6" t="str">
+        <x:v>孙雷</x:v>
+      </x:c>
+      <x:c r="B109" s="6" t="str">
+        <x:v>degree_study</x:v>
+      </x:c>
+      <x:c r="C109" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D109" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E109" s="6" t="str"/>
+      <x:c r="F109" s="6" t="str">
+        <x:v>2003</x:v>
+      </x:c>
+      <x:c r="G109" s="6" t="str"/>
+      <x:c r="H109" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I109" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J109" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K109" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L109" s="6" t="str"/>
+      <x:c r="M109" s="7" t="str"/>
+      <x:c r="N109" s="6" t="str"/>
+      <x:c r="O109" s="6" t="str">
+        <x:v>原文为本科/硕士/博士毕业，未另见明确获授学位表述；起始年月和专业未披露。</x:v>
+      </x:c>
+      <x:c r="P109" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q109" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="R109" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S109" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="64" customHeight="1">
+      <x:c r="A110" s="6" t="str">
+        <x:v>孙雷</x:v>
+      </x:c>
+      <x:c r="B110" s="6" t="str">
+        <x:v>postdoctoral_research</x:v>
+      </x:c>
+      <x:c r="C110" s="6" t="str"/>
+      <x:c r="D110" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E110" s="6" t="str">
+        <x:v>2003</x:v>
+      </x:c>
+      <x:c r="F110" s="6" t="str">
+        <x:v>2005</x:v>
+      </x:c>
+      <x:c r="G110" s="6" t="str"/>
+      <x:c r="H110" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I110" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J110" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K110" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L110" s="13" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M110" s="7" t="str"/>
+      <x:c r="N110" s="6" t="str"/>
+      <x:c r="O110" s="6" t="str">
+        <x:v>北京大学信息学院博士后，非新学位。</x:v>
+      </x:c>
+      <x:c r="P110" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q110" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="R110" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S110" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="64" customHeight="1">
+      <x:c r="A111" s="6" t="str">
+        <x:v>孙雷</x:v>
+      </x:c>
+      <x:c r="B111" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C111" s="6" t="str">
+        <x:v>副教授，硕导</x:v>
+      </x:c>
+      <x:c r="D111" s="6" t="str">
+        <x:v>北京大学集成电路学院</x:v>
+      </x:c>
+      <x:c r="E111" s="6" t="str"/>
+      <x:c r="F111" s="6" t="str"/>
+      <x:c r="G111" s="6" t="str"/>
+      <x:c r="H111" s="6" t="str"/>
+      <x:c r="I111" s="6" t="str"/>
+      <x:c r="J111" s="6" t="str"/>
+      <x:c r="K111" s="6" t="str"/>
+      <x:c r="L111" s="6" t="str"/>
+      <x:c r="M111" s="7" t="str"/>
+      <x:c r="N111" s="6" t="str"/>
+      <x:c r="O111" s="6" t="str">
+        <x:v>现行官方名录列示；不代表独立人事在岗核验，起始年月未知。</x:v>
+      </x:c>
+      <x:c r="P111" s="6" t="str"/>
+      <x:c r="Q111" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
+      </x:c>
+      <x:c r="R111" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S111" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="64" customHeight="1">
+      <x:c r="A112" s="6" t="str">
+        <x:v>孙雷</x:v>
+      </x:c>
+      <x:c r="B112" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C112" s="6" t="str">
+        <x:v>博士后</x:v>
+      </x:c>
+      <x:c r="D112" s="6" t="str">
+        <x:v>北京大学信息学院</x:v>
+      </x:c>
+      <x:c r="E112" s="6" t="str">
+        <x:v>2003</x:v>
+      </x:c>
+      <x:c r="F112" s="6" t="str">
+        <x:v>2005</x:v>
+      </x:c>
+      <x:c r="G112" s="6" t="str"/>
+      <x:c r="H112" s="6" t="str"/>
+      <x:c r="I112" s="6" t="str"/>
+      <x:c r="J112" s="6" t="str"/>
+      <x:c r="K112" s="6" t="str"/>
+      <x:c r="L112" s="6" t="str"/>
+      <x:c r="M112" s="7" t="str"/>
+      <x:c r="N112" s="6" t="str"/>
+      <x:c r="O112" s="6" t="str"/>
+      <x:c r="P112" s="6" t="str"/>
+      <x:c r="Q112" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="R112" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S112" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="64" customHeight="1">
+      <x:c r="A113" s="6" t="str">
+        <x:v>孙雷</x:v>
+      </x:c>
+      <x:c r="B113" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C113" s="6" t="str">
+        <x:v>副教授</x:v>
+      </x:c>
+      <x:c r="D113" s="6" t="str">
+        <x:v>北京大学信息学院</x:v>
+      </x:c>
+      <x:c r="E113" s="6" t="str">
+        <x:v>2005</x:v>
+      </x:c>
+      <x:c r="F113" s="6" t="str"/>
+      <x:c r="G113" s="6" t="str"/>
+      <x:c r="H113" s="6" t="str"/>
+      <x:c r="I113" s="6" t="str"/>
+      <x:c r="J113" s="6" t="str"/>
+      <x:c r="K113" s="6" t="str"/>
+      <x:c r="L113" s="6" t="str"/>
+      <x:c r="M113" s="7" t="str"/>
+      <x:c r="N113" s="6" t="str"/>
+      <x:c r="O113" s="6" t="str"/>
+      <x:c r="P113" s="6" t="str"/>
+      <x:c r="Q113" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="R113" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S113" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="64" customHeight="1">
+      <x:c r="A114" s="6" t="str">
+        <x:v>唐克超</x:v>
+      </x:c>
+      <x:c r="B114" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C114" s="6" t="str">
+        <x:v>学士</x:v>
+      </x:c>
+      <x:c r="D114" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E114" s="6" t="str">
+        <x:v>2008</x:v>
+      </x:c>
+      <x:c r="F114" s="6" t="str">
+        <x:v>2012</x:v>
+      </x:c>
+      <x:c r="G114" s="6" t="str">
+        <x:v>物理学</x:v>
+      </x:c>
+      <x:c r="H114" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I114" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J114" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K114" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L114" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M114" s="7" t="str">
+        <x:v>2012</x:v>
+      </x:c>
+      <x:c r="N114" s="6" t="str"/>
+      <x:c r="O114" s="6" t="str">
+        <x:v>院系表列学士学位；2022年Chemical Reviews作者简介明确received B.S degree。</x:v>
+      </x:c>
+      <x:c r="P114" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q114" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/tkc/index.htm</x:v>
+      </x:c>
+      <x:c r="R114" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S114" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="64" customHeight="1">
+      <x:c r="A115" s="6" t="str">
+        <x:v>唐克超</x:v>
+      </x:c>
+      <x:c r="B115" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C115" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D115" s="6" t="str">
+        <x:v>斯坦福大学</x:v>
+      </x:c>
+      <x:c r="E115" s="6" t="str">
+        <x:v>2012</x:v>
+      </x:c>
+      <x:c r="F115" s="6" t="str">
+        <x:v>2017</x:v>
+      </x:c>
+      <x:c r="G115" s="6" t="str">
+        <x:v>材料科学与工程</x:v>
+      </x:c>
+      <x:c r="H115" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="I115" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="J115" s="6" t="str">
+        <x:v>北美洲</x:v>
+      </x:c>
+      <x:c r="K115" s="6" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="L115" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M115" s="7" t="str">
+        <x:v>2017</x:v>
+      </x:c>
+      <x:c r="N115" s="6" t="str"/>
+      <x:c r="O115" s="6" t="str">
+        <x:v>院系表列博士学位；2022年Chemical Reviews作者简介明确received Ph.D degree。</x:v>
+      </x:c>
+      <x:c r="P115" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q115" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/tkc/index.htm</x:v>
+      </x:c>
+      <x:c r="R115" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S115" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="64" customHeight="1">
+      <x:c r="A116" s="6" t="str">
+        <x:v>唐克超</x:v>
+      </x:c>
+      <x:c r="B116" s="6" t="str">
+        <x:v>postdoctoral_research</x:v>
+      </x:c>
+      <x:c r="C116" s="6" t="str"/>
+      <x:c r="D116" s="6" t="str">
+        <x:v>加州大学伯克利分校</x:v>
+      </x:c>
+      <x:c r="E116" s="6" t="str">
+        <x:v>2017</x:v>
+      </x:c>
+      <x:c r="F116" s="6" t="str">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="G116" s="6" t="str"/>
+      <x:c r="H116" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="I116" s="6" t="str">
+        <x:v>美国</x:v>
+      </x:c>
+      <x:c r="J116" s="6" t="str">
+        <x:v>北美洲</x:v>
+      </x:c>
+      <x:c r="K116" s="6" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="L116" s="13" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M116" s="7" t="str"/>
+      <x:c r="N116" s="6" t="str"/>
+      <x:c r="O116" s="6" t="str"/>
+      <x:c r="P116" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q116" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/tkc/index.htm</x:v>
+      </x:c>
+      <x:c r="R116" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S116" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="64" customHeight="1">
+      <x:c r="A117" s="6" t="str">
+        <x:v>唐克超</x:v>
+      </x:c>
+      <x:c r="B117" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C117" s="6" t="str">
+        <x:v>助理教授，博导</x:v>
+      </x:c>
+      <x:c r="D117" s="6" t="str">
+        <x:v>北京大学集成电路学院</x:v>
+      </x:c>
+      <x:c r="E117" s="6" t="str"/>
+      <x:c r="F117" s="6" t="str"/>
+      <x:c r="G117" s="6" t="str"/>
+      <x:c r="H117" s="6" t="str"/>
+      <x:c r="I117" s="6" t="str"/>
+      <x:c r="J117" s="6" t="str"/>
+      <x:c r="K117" s="6" t="str"/>
+      <x:c r="L117" s="6" t="str"/>
+      <x:c r="M117" s="7" t="str"/>
+      <x:c r="N117" s="6" t="str"/>
+      <x:c r="O117" s="6" t="str">
+        <x:v>现行官方名录列示；不代表独立人事在岗核验，起始年月未知。</x:v>
+      </x:c>
+      <x:c r="P117" s="6" t="str"/>
+      <x:c r="Q117" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
+      </x:c>
+      <x:c r="R117" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S117" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="64" customHeight="1">
+      <x:c r="A118" s="6" t="str">
+        <x:v>唐克超</x:v>
+      </x:c>
+      <x:c r="B118" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C118" s="6" t="str">
+        <x:v>博士后</x:v>
+      </x:c>
+      <x:c r="D118" s="6" t="str">
+        <x:v>加州大学伯克利分校</x:v>
+      </x:c>
+      <x:c r="E118" s="6" t="str">
+        <x:v>2017</x:v>
+      </x:c>
+      <x:c r="F118" s="6" t="str">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="G118" s="6" t="str"/>
+      <x:c r="H118" s="6" t="str"/>
+      <x:c r="I118" s="6" t="str"/>
+      <x:c r="J118" s="6" t="str"/>
+      <x:c r="K118" s="6" t="str"/>
+      <x:c r="L118" s="6" t="str"/>
+      <x:c r="M118" s="7" t="str"/>
+      <x:c r="N118" s="6" t="str"/>
+      <x:c r="O118" s="6" t="str"/>
+      <x:c r="P118" s="6" t="str"/>
+      <x:c r="Q118" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/tkc/index.htm</x:v>
+      </x:c>
+      <x:c r="R118" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S118" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="64" customHeight="1">
+      <x:c r="A119" s="6" t="str">
+        <x:v>唐克超</x:v>
+      </x:c>
+      <x:c r="B119" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C119" s="6" t="str">
+        <x:v>研究员</x:v>
+      </x:c>
+      <x:c r="D119" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E119" s="6" t="str">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="F119" s="6" t="str"/>
+      <x:c r="G119" s="6" t="str"/>
+      <x:c r="H119" s="6" t="str"/>
+      <x:c r="I119" s="6" t="str"/>
+      <x:c r="J119" s="6" t="str"/>
+      <x:c r="K119" s="6" t="str"/>
+      <x:c r="L119" s="6" t="str"/>
+      <x:c r="M119" s="7" t="str"/>
+      <x:c r="N119" s="6" t="str"/>
+      <x:c r="O119" s="6" t="str">
+        <x:v>中文页头部职称为助理教授，正文工作经历为研究员；并列保存来源口径，不推断晋升日期。</x:v>
+      </x:c>
+      <x:c r="P119" s="6" t="str"/>
+      <x:c r="Q119" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/tkc/index.htm</x:v>
+      </x:c>
+      <x:c r="R119" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S119" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="64" customHeight="1">
+      <x:c r="A120" s="6" t="str">
+        <x:v>王宗巍</x:v>
+      </x:c>
+      <x:c r="B120" s="6" t="str">
+        <x:v>degree_study</x:v>
+      </x:c>
+      <x:c r="C120" s="6" t="str">
+        <x:v>本科</x:v>
+      </x:c>
+      <x:c r="D120" s="6" t="str">
+        <x:v>西安电子科技大学</x:v>
+      </x:c>
+      <x:c r="E120" s="6" t="str"/>
+      <x:c r="F120" s="6" t="str"/>
+      <x:c r="G120" s="6" t="str"/>
+      <x:c r="H120" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I120" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J120" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K120" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L120" s="6" t="str"/>
+      <x:c r="M120" s="7" t="str"/>
+      <x:c r="N120" s="6" t="str"/>
+      <x:c r="O120" s="6" t="str">
+        <x:v>官方页只述毕业院校及学历阶段，未给明确授位、时间或专业；不以博导职务证明本人获博士。</x:v>
+      </x:c>
+      <x:c r="P120" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q120" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wzw/index.htm</x:v>
+      </x:c>
+      <x:c r="R120" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S120" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="64" customHeight="1">
+      <x:c r="A121" s="6" t="str">
+        <x:v>王宗巍</x:v>
+      </x:c>
+      <x:c r="B121" s="6" t="str">
+        <x:v>degree_study</x:v>
+      </x:c>
+      <x:c r="C121" s="6" t="str">
+        <x:v>硕士</x:v>
+      </x:c>
+      <x:c r="D121" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E121" s="6" t="str"/>
+      <x:c r="F121" s="6" t="str"/>
+      <x:c r="G121" s="6" t="str"/>
+      <x:c r="H121" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I121" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J121" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K121" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L121" s="6" t="str"/>
+      <x:c r="M121" s="7" t="str"/>
+      <x:c r="N121" s="6" t="str"/>
+      <x:c r="O121" s="6" t="str">
+        <x:v>官方页只述毕业院校及学历阶段，未给明确授位、时间或专业；不以博导职务证明本人获博士。</x:v>
+      </x:c>
+      <x:c r="P121" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q121" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wzw/index.htm</x:v>
+      </x:c>
+      <x:c r="R121" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S121" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="64" customHeight="1">
+      <x:c r="A122" s="6" t="str">
+        <x:v>王宗巍</x:v>
+      </x:c>
+      <x:c r="B122" s="6" t="str">
+        <x:v>degree_study</x:v>
+      </x:c>
+      <x:c r="C122" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D122" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E122" s="6" t="str"/>
+      <x:c r="F122" s="6" t="str"/>
+      <x:c r="G122" s="6" t="str"/>
+      <x:c r="H122" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I122" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J122" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K122" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L122" s="6" t="str"/>
+      <x:c r="M122" s="7" t="str"/>
+      <x:c r="N122" s="6" t="str"/>
+      <x:c r="O122" s="6" t="str">
+        <x:v>官方页只述毕业院校及学历阶段，未给明确授位、时间或专业；不以博导职务证明本人获博士。</x:v>
+      </x:c>
+      <x:c r="P122" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q122" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wzw/index.htm</x:v>
+      </x:c>
+      <x:c r="R122" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S122" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="64" customHeight="1">
+      <x:c r="A123" s="6" t="str">
+        <x:v>王宗巍</x:v>
+      </x:c>
+      <x:c r="B123" s="6" t="str">
+        <x:v>postdoctoral_research</x:v>
+      </x:c>
+      <x:c r="C123" s="6" t="str"/>
+      <x:c r="D123" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E123" s="6" t="str"/>
+      <x:c r="F123" s="6" t="str"/>
+      <x:c r="G123" s="6" t="str"/>
+      <x:c r="H123" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I123" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J123" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K123" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L123" s="13" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M123" s="7" t="str"/>
+      <x:c r="N123" s="6" t="str"/>
+      <x:c r="O123" s="6" t="str">
+        <x:v>工作表2018–2021为博士后/讲师、助理研究员合并区间；博士后独立起止不详，不套用整个合并区间。</x:v>
+      </x:c>
+      <x:c r="P123" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q123" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wzw/index.htm</x:v>
+      </x:c>
+      <x:c r="R123" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S123" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="64" customHeight="1">
+      <x:c r="A124" s="6" t="str">
+        <x:v>王宗巍</x:v>
+      </x:c>
+      <x:c r="B124" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C124" s="6" t="str">
+        <x:v>助理教授、博导</x:v>
+      </x:c>
+      <x:c r="D124" s="6" t="str">
+        <x:v>北京大学集成电路学院</x:v>
+      </x:c>
+      <x:c r="E124" s="6" t="str"/>
+      <x:c r="F124" s="6" t="str"/>
+      <x:c r="G124" s="6" t="str"/>
+      <x:c r="H124" s="6" t="str"/>
+      <x:c r="I124" s="6" t="str"/>
+      <x:c r="J124" s="6" t="str"/>
+      <x:c r="K124" s="6" t="str"/>
+      <x:c r="L124" s="6" t="str"/>
+      <x:c r="M124" s="7" t="str"/>
+      <x:c r="N124" s="6" t="str"/>
+      <x:c r="O124" s="6" t="str">
+        <x:v>现行官方名录列示；不代表独立人事在岗核验，起始年月未知。</x:v>
+      </x:c>
+      <x:c r="P124" s="6" t="str"/>
+      <x:c r="Q124" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
+      </x:c>
+      <x:c r="R124" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S124" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="64" customHeight="1">
+      <x:c r="A125" s="6" t="str">
+        <x:v>王宗巍</x:v>
+      </x:c>
+      <x:c r="B125" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C125" s="6" t="str">
+        <x:v>博士后/讲师、助理研究员</x:v>
+      </x:c>
+      <x:c r="D125" s="6" t="str">
+        <x:v>北京大学信息科学技术学院</x:v>
+      </x:c>
+      <x:c r="E125" s="6" t="str">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="F125" s="6" t="str">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="G125" s="6" t="str"/>
+      <x:c r="H125" s="6" t="str"/>
+      <x:c r="I125" s="6" t="str"/>
+      <x:c r="J125" s="6" t="str"/>
+      <x:c r="K125" s="6" t="str"/>
+      <x:c r="L125" s="6" t="str"/>
+      <x:c r="M125" s="7" t="str"/>
+      <x:c r="N125" s="6" t="str"/>
+      <x:c r="O125" s="6" t="str">
+        <x:v>官网合并区间，不拆造各岗位起讫。</x:v>
+      </x:c>
+      <x:c r="P125" s="6" t="str"/>
+      <x:c r="Q125" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wzw/index.htm</x:v>
+      </x:c>
+      <x:c r="R125" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S125" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="64" customHeight="1">
+      <x:c r="A126" s="6" t="str">
+        <x:v>王宗巍</x:v>
+      </x:c>
+      <x:c r="B126" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C126" s="6" t="str">
+        <x:v>助理研究员，副研究员、研究员/博士生导师</x:v>
+      </x:c>
+      <x:c r="D126" s="6" t="str">
+        <x:v>北京大学集成电路学院</x:v>
+      </x:c>
+      <x:c r="E126" s="6" t="str">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="F126" s="6" t="str"/>
+      <x:c r="G126" s="6" t="str"/>
+      <x:c r="H126" s="6" t="str"/>
+      <x:c r="I126" s="6" t="str"/>
+      <x:c r="J126" s="6" t="str"/>
+      <x:c r="K126" s="6" t="str"/>
+      <x:c r="L126" s="6" t="str"/>
+      <x:c r="M126" s="7" t="str"/>
+      <x:c r="N126" s="6" t="str"/>
+      <x:c r="O126" s="6" t="str">
+        <x:v>官网正文合并岗位，头部助理教授；不拆造职称变动时间。</x:v>
+      </x:c>
+      <x:c r="P126" s="6" t="str"/>
+      <x:c r="Q126" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wzw/index.htm</x:v>
+      </x:c>
+      <x:c r="R126" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S126" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="64" customHeight="1">
+      <x:c r="A127" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B127" s="6" t="str">
+        <x:v>degree_study</x:v>
+      </x:c>
+      <x:c r="C127" s="6" t="str">
+        <x:v>本科</x:v>
+      </x:c>
+      <x:c r="D127" s="6" t="str">
+        <x:v>西安电子科技大学</x:v>
+      </x:c>
+      <x:c r="E127" s="6" t="str">
+        <x:v>1989-09</x:v>
+      </x:c>
+      <x:c r="F127" s="6" t="str">
+        <x:v>1993-06</x:v>
+      </x:c>
+      <x:c r="G127" s="6" t="str"/>
+      <x:c r="H127" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I127" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J127" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K127" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L127" s="6" t="str"/>
+      <x:c r="M127" s="7" t="str"/>
+      <x:c r="N127" s="6" t="str"/>
+      <x:c r="O127" s="6" t="str">
+        <x:v>官网学历阶段标签，未另见明确获授学位表述。</x:v>
+      </x:c>
+      <x:c r="P127" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q127" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="R127" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S127" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="64" customHeight="1">
+      <x:c r="A128" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B128" s="6" t="str">
+        <x:v>degree_study</x:v>
+      </x:c>
+      <x:c r="C128" s="6" t="str">
+        <x:v>硕士</x:v>
+      </x:c>
+      <x:c r="D128" s="6" t="str">
+        <x:v>西安电子科技大学</x:v>
+      </x:c>
+      <x:c r="E128" s="6" t="str">
+        <x:v>1993-09</x:v>
+      </x:c>
+      <x:c r="F128" s="6" t="str">
+        <x:v>1996-07</x:v>
+      </x:c>
+      <x:c r="G128" s="6" t="str"/>
+      <x:c r="H128" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I128" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J128" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K128" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L128" s="6" t="str"/>
+      <x:c r="M128" s="7" t="str"/>
+      <x:c r="N128" s="6" t="str"/>
+      <x:c r="O128" s="6" t="str">
+        <x:v>官网学历阶段标签，未另见明确获授学位表述。</x:v>
+      </x:c>
+      <x:c r="P128" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q128" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="R128" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S128" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="64" customHeight="1">
+      <x:c r="A129" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B129" s="6" t="str">
+        <x:v>degree</x:v>
+      </x:c>
+      <x:c r="C129" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D129" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E129" s="6" t="str">
+        <x:v>1996-09</x:v>
+      </x:c>
+      <x:c r="F129" s="6" t="str">
+        <x:v>2000-03</x:v>
+      </x:c>
+      <x:c r="G129" s="6" t="str"/>
+      <x:c r="H129" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I129" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J129" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K129" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L129" s="13" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M129" s="7" t="str">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="N129" s="6" t="str"/>
+      <x:c r="O129" s="6" t="str">
+        <x:v>博士由北大官方旧系介绍第5页明确2000年获理学博士学位；其余仅学习标签，未推授位。</x:v>
+      </x:c>
+      <x:c r="P129" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q129" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="R129" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S129" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="64" customHeight="1">
+      <x:c r="A130" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B130" s="6" t="str">
+        <x:v>postdoctoral_research</x:v>
+      </x:c>
+      <x:c r="C130" s="6" t="str"/>
+      <x:c r="D130" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E130" s="6" t="str">
+        <x:v>2000-04</x:v>
+      </x:c>
+      <x:c r="F130" s="6" t="str">
+        <x:v>2002-03</x:v>
+      </x:c>
+      <x:c r="G130" s="6" t="str"/>
+      <x:c r="H130" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I130" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J130" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K130" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L130" s="13" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M130" s="7" t="str"/>
+      <x:c r="N130" s="6" t="str"/>
+      <x:c r="O130" s="6" t="str"/>
+      <x:c r="P130" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q130" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="R130" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S130" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="64" customHeight="1">
+      <x:c r="A131" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B131" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C131" s="6" t="str">
+        <x:v>教授，博导</x:v>
+      </x:c>
+      <x:c r="D131" s="6" t="str">
+        <x:v>北京大学集成电路学院</x:v>
+      </x:c>
+      <x:c r="E131" s="6" t="str"/>
+      <x:c r="F131" s="6" t="str"/>
+      <x:c r="G131" s="6" t="str"/>
+      <x:c r="H131" s="6" t="str"/>
+      <x:c r="I131" s="6" t="str"/>
+      <x:c r="J131" s="6" t="str"/>
+      <x:c r="K131" s="6" t="str"/>
+      <x:c r="L131" s="6" t="str"/>
+      <x:c r="M131" s="7" t="str"/>
+      <x:c r="N131" s="6" t="str"/>
+      <x:c r="O131" s="6" t="str">
+        <x:v>现行官方名录列示；不代表独立人事在岗核验，起始年月未知。</x:v>
+      </x:c>
+      <x:c r="P131" s="6" t="str"/>
+      <x:c r="Q131" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
+      </x:c>
+      <x:c r="R131" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S131" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="64" customHeight="1">
+      <x:c r="A132" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B132" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C132" s="6" t="str">
+        <x:v>博士后</x:v>
+      </x:c>
+      <x:c r="D132" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E132" s="6" t="str">
+        <x:v>2000-04</x:v>
+      </x:c>
+      <x:c r="F132" s="6" t="str">
+        <x:v>2002-03</x:v>
+      </x:c>
+      <x:c r="G132" s="6" t="str"/>
+      <x:c r="H132" s="6" t="str"/>
+      <x:c r="I132" s="6" t="str"/>
+      <x:c r="J132" s="6" t="str"/>
+      <x:c r="K132" s="6" t="str"/>
+      <x:c r="L132" s="6" t="str"/>
+      <x:c r="M132" s="7" t="str"/>
+      <x:c r="N132" s="6" t="str"/>
+      <x:c r="O132" s="6" t="str"/>
+      <x:c r="P132" s="6" t="str"/>
+      <x:c r="Q132" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="R132" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S132" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="64" customHeight="1">
+      <x:c r="A133" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B133" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C133" s="6" t="str">
+        <x:v>讲师，副教授，教授</x:v>
+      </x:c>
+      <x:c r="D133" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E133" s="6" t="str">
+        <x:v>2002-04</x:v>
+      </x:c>
+      <x:c r="F133" s="6" t="str"/>
+      <x:c r="G133" s="6" t="str"/>
+      <x:c r="H133" s="6" t="str"/>
+      <x:c r="I133" s="6" t="str"/>
+      <x:c r="J133" s="6" t="str"/>
+      <x:c r="K133" s="6" t="str"/>
+      <x:c r="L133" s="6" t="str"/>
+      <x:c r="M133" s="7" t="str"/>
+      <x:c r="N133" s="6" t="str"/>
+      <x:c r="O133" s="6" t="str">
+        <x:v>官网合并工作区间，不把起始月当教授晋升日期。</x:v>
+      </x:c>
+      <x:c r="P133" s="6" t="str"/>
+      <x:c r="Q133" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="R133" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S133" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="64" customHeight="1">
+      <x:c r="A134" s="6" t="str">
+        <x:v>王茂俊</x:v>
+      </x:c>
+      <x:c r="B134" s="6" t="str">
+        <x:v>degree_study</x:v>
+      </x:c>
+      <x:c r="C134" s="6" t="str">
+        <x:v>学士</x:v>
+      </x:c>
+      <x:c r="D134" s="6" t="str">
+        <x:v>南京大学</x:v>
+      </x:c>
+      <x:c r="E134" s="6" t="str">
+        <x:v>1998-09</x:v>
+      </x:c>
+      <x:c r="F134" s="6" t="str">
+        <x:v>2002-07</x:v>
+      </x:c>
+      <x:c r="G134" s="6" t="str">
+        <x:v>物理</x:v>
+      </x:c>
+      <x:c r="H134" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I134" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J134" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K134" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L134" s="6" t="str"/>
+      <x:c r="M134" s="7" t="str"/>
+      <x:c r="N134" s="6" t="str"/>
+      <x:c r="O134" s="6" t="str">
+        <x:v>强化部学士标签，未另见明确获授学位表述。</x:v>
+      </x:c>
+      <x:c r="P134" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q134" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wmj/index.htm</x:v>
+      </x:c>
+      <x:c r="R134" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S134" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="64" customHeight="1">
+      <x:c r="A135" s="6" t="str">
+        <x:v>王茂俊</x:v>
+      </x:c>
+      <x:c r="B135" s="6" t="str">
+        <x:v>degree_study</x:v>
+      </x:c>
+      <x:c r="C135" s="6" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D135" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+      <x:c r="E135" s="6" t="str">
+        <x:v>2002-09</x:v>
+      </x:c>
+      <x:c r="F135" s="6" t="str">
+        <x:v>2007-07</x:v>
+      </x:c>
+      <x:c r="G135" s="6" t="str">
+        <x:v>半导体光电子学</x:v>
+      </x:c>
+      <x:c r="H135" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I135" s="6" t="str">
+        <x:v>中国内地</x:v>
+      </x:c>
+      <x:c r="J135" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K135" s="6" t="str">
+        <x:v>unknown</x:v>
+      </x:c>
+      <x:c r="L135" s="6" t="str"/>
+      <x:c r="M135" s="7" t="str"/>
+      <x:c r="N135" s="6" t="str"/>
+      <x:c r="O135" s="6" t="str">
+        <x:v>物理系博士标签，未另见已读取官方授位陈述。</x:v>
+      </x:c>
+      <x:c r="P135" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q135" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wmj/index.htm</x:v>
+      </x:c>
+      <x:c r="R135" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S135" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="64" customHeight="1">
+      <x:c r="A136" s="6" t="str">
+        <x:v>王茂俊</x:v>
+      </x:c>
+      <x:c r="B136" s="6" t="str">
+        <x:v>postdoctoral_research</x:v>
+      </x:c>
+      <x:c r="C136" s="6" t="str"/>
+      <x:c r="D136" s="6" t="str">
+        <x:v>香港科技大学</x:v>
+      </x:c>
+      <x:c r="E136" s="6" t="str">
+        <x:v>2007-08</x:v>
+      </x:c>
+      <x:c r="F136" s="6" t="str">
+        <x:v>2009-12</x:v>
+      </x:c>
+      <x:c r="G136" s="6" t="str"/>
+      <x:c r="H136" s="6" t="str">
+        <x:v>中国</x:v>
+      </x:c>
+      <x:c r="I136" s="6" t="str">
+        <x:v>中国香港</x:v>
+      </x:c>
+      <x:c r="J136" s="6" t="str">
+        <x:v>亚洲</x:v>
+      </x:c>
+      <x:c r="K136" s="6" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="L136" s="13" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M136" s="7" t="str"/>
+      <x:c r="N136" s="6" t="str"/>
+      <x:c r="O136" s="6" t="str"/>
+      <x:c r="P136" s="6" t="str">
+        <x:v>按来源所指院校所在地标准化，不代表国籍；授位地点与访问、攻读未获学位、联合培养分开。</x:v>
+      </x:c>
+      <x:c r="Q136" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wmj/index.htm</x:v>
+      </x:c>
+      <x:c r="R136" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S136" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="64" customHeight="1">
+      <x:c r="A137" s="6" t="str">
+        <x:v>王茂俊</x:v>
+      </x:c>
+      <x:c r="B137" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C137" s="6" t="str">
+        <x:v>副教授，博导</x:v>
+      </x:c>
+      <x:c r="D137" s="6" t="str">
+        <x:v>北京大学集成电路学院</x:v>
+      </x:c>
+      <x:c r="E137" s="6" t="str"/>
+      <x:c r="F137" s="6" t="str"/>
+      <x:c r="G137" s="6" t="str"/>
+      <x:c r="H137" s="6" t="str"/>
+      <x:c r="I137" s="6" t="str"/>
+      <x:c r="J137" s="6" t="str"/>
+      <x:c r="K137" s="6" t="str"/>
+      <x:c r="L137" s="6" t="str"/>
+      <x:c r="M137" s="7" t="str"/>
+      <x:c r="N137" s="6" t="str"/>
+      <x:c r="O137" s="6" t="str">
+        <x:v>现行官方名录列示；不代表独立人事在岗核验，起始年月未知。</x:v>
+      </x:c>
+      <x:c r="P137" s="6" t="str"/>
+      <x:c r="Q137" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
+      </x:c>
+      <x:c r="R137" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S137" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="64" customHeight="1">
+      <x:c r="A138" s="6" t="str">
+        <x:v>王茂俊</x:v>
+      </x:c>
+      <x:c r="B138" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C138" s="6" t="str">
+        <x:v>博士后</x:v>
+      </x:c>
+      <x:c r="D138" s="6" t="str">
+        <x:v>香港科技大学电子和计算机工程系</x:v>
+      </x:c>
+      <x:c r="E138" s="6" t="str">
+        <x:v>2007-08</x:v>
+      </x:c>
+      <x:c r="F138" s="6" t="str">
+        <x:v>2009-12</x:v>
+      </x:c>
+      <x:c r="G138" s="6" t="str"/>
+      <x:c r="H138" s="6" t="str"/>
+      <x:c r="I138" s="6" t="str"/>
+      <x:c r="J138" s="6" t="str"/>
+      <x:c r="K138" s="6" t="str"/>
+      <x:c r="L138" s="6" t="str"/>
+      <x:c r="M138" s="7" t="str"/>
+      <x:c r="N138" s="6" t="str"/>
+      <x:c r="O138" s="6" t="str"/>
+      <x:c r="P138" s="6" t="str"/>
+      <x:c r="Q138" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wmj/index.htm</x:v>
+      </x:c>
+      <x:c r="R138" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S138" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="64" customHeight="1">
+      <x:c r="A139" s="6" t="str">
+        <x:v>王茂俊</x:v>
+      </x:c>
+      <x:c r="B139" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C139" s="6" t="str">
+        <x:v>工程师</x:v>
+      </x:c>
+      <x:c r="D139" s="6" t="str">
+        <x:v>南京电子器件研究所宽禁带半导体研发部</x:v>
+      </x:c>
+      <x:c r="E139" s="6" t="str">
+        <x:v>2010-01</x:v>
+      </x:c>
+      <x:c r="F139" s="6" t="str">
+        <x:v>2010-07</x:v>
+      </x:c>
+      <x:c r="G139" s="6" t="str"/>
+      <x:c r="H139" s="6" t="str"/>
+      <x:c r="I139" s="6" t="str"/>
+      <x:c r="J139" s="6" t="str"/>
+      <x:c r="K139" s="6" t="str"/>
+      <x:c r="L139" s="6" t="str"/>
+      <x:c r="M139" s="7" t="str"/>
+      <x:c r="N139" s="6" t="str"/>
+      <x:c r="O139" s="6" t="str"/>
+      <x:c r="P139" s="6" t="str"/>
+      <x:c r="Q139" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wmj/index.htm</x:v>
+      </x:c>
+      <x:c r="R139" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S139" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="64" customHeight="1">
+      <x:c r="A140" s="6" t="str">
+        <x:v>王茂俊</x:v>
+      </x:c>
+      <x:c r="B140" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C140" s="6" t="str">
+        <x:v>讲师</x:v>
+      </x:c>
+      <x:c r="D140" s="6" t="str">
+        <x:v>北京大学信息科学技术学院微纳电子学系</x:v>
+      </x:c>
+      <x:c r="E140" s="6" t="str">
+        <x:v>2011-08</x:v>
+      </x:c>
+      <x:c r="F140" s="6" t="str">
+        <x:v>2013-07</x:v>
+      </x:c>
+      <x:c r="G140" s="6" t="str"/>
+      <x:c r="H140" s="6" t="str"/>
+      <x:c r="I140" s="6" t="str"/>
+      <x:c r="J140" s="6" t="str"/>
+      <x:c r="K140" s="6" t="str"/>
+      <x:c r="L140" s="6" t="str"/>
+      <x:c r="M140" s="7" t="str"/>
+      <x:c r="N140" s="6" t="str"/>
+      <x:c r="O140" s="6" t="str"/>
+      <x:c r="P140" s="6" t="str"/>
+      <x:c r="Q140" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wmj/index.htm</x:v>
+      </x:c>
+      <x:c r="R140" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S140" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="64" customHeight="1">
+      <x:c r="A141" s="6" t="str">
+        <x:v>王茂俊</x:v>
+      </x:c>
+      <x:c r="B141" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C141" s="6" t="str">
+        <x:v>副教授</x:v>
+      </x:c>
+      <x:c r="D141" s="6" t="str">
+        <x:v>北京大学信息科学技术学院微纳电子学系</x:v>
+      </x:c>
+      <x:c r="E141" s="6" t="str">
+        <x:v>2013-08</x:v>
+      </x:c>
+      <x:c r="F141" s="6" t="str">
+        <x:v>2021-04</x:v>
+      </x:c>
+      <x:c r="G141" s="6" t="str"/>
+      <x:c r="H141" s="6" t="str"/>
+      <x:c r="I141" s="6" t="str"/>
+      <x:c r="J141" s="6" t="str"/>
+      <x:c r="K141" s="6" t="str"/>
+      <x:c r="L141" s="6" t="str"/>
+      <x:c r="M141" s="7" t="str"/>
+      <x:c r="N141" s="6" t="str"/>
+      <x:c r="O141" s="6" t="str"/>
+      <x:c r="P141" s="6" t="str"/>
+      <x:c r="Q141" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wmj/index.htm</x:v>
+      </x:c>
+      <x:c r="R141" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S141" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="64" customHeight="1">
+      <x:c r="A142" s="6" t="str">
+        <x:v>王茂俊</x:v>
+      </x:c>
+      <x:c r="B142" s="6" t="str">
+        <x:v>employment</x:v>
+      </x:c>
+      <x:c r="C142" s="6" t="str">
+        <x:v>副教授</x:v>
+      </x:c>
+      <x:c r="D142" s="6" t="str">
+        <x:v>北京大学集成电路学院</x:v>
+      </x:c>
+      <x:c r="E142" s="6" t="str">
+        <x:v>2021-05</x:v>
+      </x:c>
+      <x:c r="F142" s="6" t="str"/>
+      <x:c r="G142" s="6" t="str"/>
+      <x:c r="H142" s="6" t="str"/>
+      <x:c r="I142" s="6" t="str"/>
+      <x:c r="J142" s="6" t="str"/>
+      <x:c r="K142" s="6" t="str"/>
+      <x:c r="L142" s="6" t="str"/>
+      <x:c r="M142" s="7" t="str"/>
+      <x:c r="N142" s="6" t="str"/>
+      <x:c r="O142" s="6" t="str"/>
+      <x:c r="P142" s="6" t="str"/>
+      <x:c r="Q142" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wmj/index.htm</x:v>
+      </x:c>
+      <x:c r="R142" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="S142" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e74c69a378848f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda35436a63d84555"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4695,7 +8022,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2d02a1a17f44209"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9a9d612601e48b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5542,10 +8869,372 @@
         <x:v>北京大学</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="64" customHeight="1">
+      <x:c r="A23" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B23" s="6" t="str">
+        <x:v>In-memory analog solution of compressed sensing recovery in one step</x:v>
+      </x:c>
+      <x:c r="C23" s="6" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="D23" s="6" t="str"/>
+      <x:c r="E23" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="F23" s="6" t="str">
+        <x:v>journal_article</x:v>
+      </x:c>
+      <x:c r="G23" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="H23" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="I23" s="6" t="str">
+        <x:v>official_publication_list_only</x:v>
+      </x:c>
+      <x:c r="J23" s="6" t="str">
+        <x:v>官网精选条目，未逐篇查出版者或补DOI。</x:v>
+      </x:c>
+      <x:c r="K23" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="L23" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="64" customHeight="1">
+      <x:c r="A24" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B24" s="6" t="str">
+        <x:v>A full spectrum of computing-in-memory technologies</x:v>
+      </x:c>
+      <x:c r="C24" s="6" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="D24" s="6" t="str"/>
+      <x:c r="E24" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="F24" s="6" t="str">
+        <x:v>journal_article</x:v>
+      </x:c>
+      <x:c r="G24" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="H24" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="I24" s="6" t="str">
+        <x:v>official_publication_list_only</x:v>
+      </x:c>
+      <x:c r="J24" s="6" t="str">
+        <x:v>官网精选条目，未逐篇查出版者或补DOI。</x:v>
+      </x:c>
+      <x:c r="K24" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="L24" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="64" customHeight="1">
+      <x:c r="A25" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B25" s="6" t="str">
+        <x:v>Extremely-Fast, Energy-Efficient Massive MIMO Precoding with Analog RRAM Matrix Computing</x:v>
+      </x:c>
+      <x:c r="C25" s="6" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="D25" s="6" t="str"/>
+      <x:c r="E25" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="F25" s="6" t="str">
+        <x:v>journal_article</x:v>
+      </x:c>
+      <x:c r="G25" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="H25" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="I25" s="6" t="str">
+        <x:v>official_publication_list_only</x:v>
+      </x:c>
+      <x:c r="J25" s="6" t="str">
+        <x:v>官网精选条目，未逐篇查出版者或补DOI。</x:v>
+      </x:c>
+      <x:c r="K25" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="L25" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="64" customHeight="1">
+      <x:c r="A26" s="6" t="str">
+        <x:v>孙雷</x:v>
+      </x:c>
+      <x:c r="B26" s="6" t="str">
+        <x:v>Impact of gate coupling and misalignment on performance of double-gate organic thin film transistors</x:v>
+      </x:c>
+      <x:c r="C26" s="6" t="n">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="D26" s="6" t="str"/>
+      <x:c r="E26" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="F26" s="6" t="str">
+        <x:v>journal_article</x:v>
+      </x:c>
+      <x:c r="G26" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="H26" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="I26" s="6" t="str">
+        <x:v>official_publication_list_only</x:v>
+      </x:c>
+      <x:c r="J26" s="6" t="str">
+        <x:v>本人官方主页列示，未逐篇核验出版者或补猜DOI。</x:v>
+      </x:c>
+      <x:c r="K26" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="L26" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="64" customHeight="1">
+      <x:c r="A27" s="6" t="str">
+        <x:v>孙雷</x:v>
+      </x:c>
+      <x:c r="B27" s="6" t="str">
+        <x:v>Comparative study of silicon nanowire transistors with triangular-shaped cross sections</x:v>
+      </x:c>
+      <x:c r="C27" s="6" t="n">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="D27" s="6" t="str"/>
+      <x:c r="E27" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="F27" s="6" t="str">
+        <x:v>journal_article</x:v>
+      </x:c>
+      <x:c r="G27" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="H27" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="I27" s="6" t="str">
+        <x:v>official_publication_list_only</x:v>
+      </x:c>
+      <x:c r="J27" s="6" t="str">
+        <x:v>本人官方主页列示，未逐篇核验出版者或补猜DOI。</x:v>
+      </x:c>
+      <x:c r="K27" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="L27" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="64" customHeight="1">
+      <x:c r="A28" s="6" t="str">
+        <x:v>孙雷</x:v>
+      </x:c>
+      <x:c r="B28" s="6" t="str">
+        <x:v>Simulation and comparative study of tunneling field effect transistors with dopant-segregated Schottky source/drain</x:v>
+      </x:c>
+      <x:c r="C28" s="6" t="n">
+        <x:v>2016</x:v>
+      </x:c>
+      <x:c r="D28" s="6" t="str"/>
+      <x:c r="E28" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="F28" s="6" t="str">
+        <x:v>journal_article</x:v>
+      </x:c>
+      <x:c r="G28" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="H28" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="I28" s="6" t="str">
+        <x:v>official_publication_list_only</x:v>
+      </x:c>
+      <x:c r="J28" s="6" t="str">
+        <x:v>本人官方主页列示，未逐篇核验出版者或补猜DOI。</x:v>
+      </x:c>
+      <x:c r="K28" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="L28" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="64" customHeight="1">
+      <x:c r="A29" s="6" t="str">
+        <x:v>唐克超</x:v>
+      </x:c>
+      <x:c r="B29" s="6" t="str">
+        <x:v>Enabling Active Nanotechnologies by Phase Transition: From Electronics, Photonics to Thermotics</x:v>
+      </x:c>
+      <x:c r="C29" s="6" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="D29" s="6" t="str">
+        <x:v>10.1021/acs.chemrev.2c00171</x:v>
+      </x:c>
+      <x:c r="E29" s="6" t="str">
+        <x:v>https://doi.org/10.1021/acs.chemrev.2c00171</x:v>
+      </x:c>
+      <x:c r="F29" s="6" t="str">
+        <x:v>review_article</x:v>
+      </x:c>
+      <x:c r="G29" s="6" t="str">
+        <x:v>https://wu.mse.berkeley.edu/publications/Qiu-ChemRev2022.pdf</x:v>
+      </x:c>
+      <x:c r="H29" s="6" t="str">
+        <x:v>https://wu.mse.berkeley.edu/publications/Qiu-ChemRev2022.pdf</x:v>
+      </x:c>
+      <x:c r="I29" s="6" t="str">
+        <x:v>article_metadata_verified</x:v>
+      </x:c>
+      <x:c r="J29" s="6" t="str">
+        <x:v>大学官方课题组托管的出版者PDF，标题、作者及本人简介均已核。</x:v>
+      </x:c>
+      <x:c r="K29" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="L29" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="64" customHeight="1">
+      <x:c r="A30" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B30" s="6" t="str">
+        <x:v>Investigation on mechanisms of current saturation in gateless AlGaN/GaN heterostructure device</x:v>
+      </x:c>
+      <x:c r="C30" s="6" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="D30" s="6" t="str"/>
+      <x:c r="E30" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="F30" s="6" t="str">
+        <x:v>journal_article</x:v>
+      </x:c>
+      <x:c r="G30" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="H30" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="I30" s="6" t="str">
+        <x:v>official_publication_list_only</x:v>
+      </x:c>
+      <x:c r="J30" s="6" t="str">
+        <x:v>本人官方主页精选条目，未逐篇核验出版者或补猜DOI。</x:v>
+      </x:c>
+      <x:c r="K30" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="L30" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="64" customHeight="1">
+      <x:c r="A31" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B31" s="6" t="str">
+        <x:v>Improved fabrication of fully-recessed normally-off SiN/SiO2/GaN MISFET based on the self-terminated gate recess etching technique</x:v>
+      </x:c>
+      <x:c r="C31" s="6" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="D31" s="6" t="str"/>
+      <x:c r="E31" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="F31" s="6" t="str">
+        <x:v>journal_article</x:v>
+      </x:c>
+      <x:c r="G31" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="H31" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="I31" s="6" t="str">
+        <x:v>official_publication_list_only</x:v>
+      </x:c>
+      <x:c r="J31" s="6" t="str">
+        <x:v>本人官方主页精选条目，未逐篇核验出版者或补猜DOI。</x:v>
+      </x:c>
+      <x:c r="K31" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="L31" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="64" customHeight="1">
+      <x:c r="A32" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B32" s="6" t="str">
+        <x:v>Study on the charging current of surface traps in AlGaN/GaN high electron mobility transistors with a slot gate structure</x:v>
+      </x:c>
+      <x:c r="C32" s="6" t="n">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="D32" s="6" t="str"/>
+      <x:c r="E32" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="F32" s="6" t="str">
+        <x:v>journal_article</x:v>
+      </x:c>
+      <x:c r="G32" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="H32" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="I32" s="6" t="str">
+        <x:v>official_publication_list_only</x:v>
+      </x:c>
+      <x:c r="J32" s="6" t="str">
+        <x:v>本人官方主页精选条目，未逐篇核验出版者或补猜DOI。</x:v>
+      </x:c>
+      <x:c r="K32" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="L32" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52d435bd892740a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92de7408e3134533"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7612,16 +11301,16 @@
     </x:row>
     <x:row r="90" ht="64" customHeight="1">
       <x:c r="A90" s="6" t="str">
-        <x:v>蔡一茂</x:v>
+        <x:v>黎明</x:v>
       </x:c>
       <x:c r="B90" s="6" t="str">
-        <x:v>institution-classification-8</x:v>
+        <x:v>liming-source-1</x:v>
       </x:c>
       <x:c r="C90" s="6" t="str">
-        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
       </x:c>
       <x:c r="D90" s="6" t="str">
-        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+        <x:v>official_roster_read</x:v>
       </x:c>
       <x:c r="E90" s="7" t="d">
         <x:v>2026-10-23T00:00:00.000Z</x:v>
@@ -7635,16 +11324,16 @@
     </x:row>
     <x:row r="91" ht="64" customHeight="1">
       <x:c r="A91" s="6" t="str">
-        <x:v>程哲</x:v>
+        <x:v>黎明</x:v>
       </x:c>
       <x:c r="B91" s="6" t="str">
-        <x:v>institution-classification-14</x:v>
+        <x:v>liming-source-2</x:v>
       </x:c>
       <x:c r="C91" s="6" t="str">
-        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/lm/index.htm</x:v>
       </x:c>
       <x:c r="D91" s="6" t="str">
-        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+        <x:v>official_publisher_or_institution_metadata</x:v>
       </x:c>
       <x:c r="E91" s="7" t="d">
         <x:v>2026-10-23T00:00:00.000Z</x:v>
@@ -7658,16 +11347,16 @@
     </x:row>
     <x:row r="92" ht="64" customHeight="1">
       <x:c r="A92" s="6" t="str">
-        <x:v>傅云义</x:v>
+        <x:v>刘力锋</x:v>
       </x:c>
       <x:c r="B92" s="6" t="str">
-        <x:v>institution-classification-6</x:v>
+        <x:v>liulifeng-source-1</x:v>
       </x:c>
       <x:c r="C92" s="6" t="str">
-        <x:v>https://www.csust.edu.cn/fzgh/info/1016/1662.htm</x:v>
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
       </x:c>
       <x:c r="D92" s="6" t="str">
-        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+        <x:v>official_roster_read</x:v>
       </x:c>
       <x:c r="E92" s="7" t="d">
         <x:v>2026-10-23T00:00:00.000Z</x:v>
@@ -7681,16 +11370,16 @@
     </x:row>
     <x:row r="93" ht="64" customHeight="1">
       <x:c r="A93" s="6" t="str">
-        <x:v>贺明</x:v>
+        <x:v>刘力锋</x:v>
       </x:c>
       <x:c r="B93" s="6" t="str">
-        <x:v>institution-classification-8</x:v>
+        <x:v>liulifeng-source-2</x:v>
       </x:c>
       <x:c r="C93" s="6" t="str">
-        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/llf/index.htm</x:v>
       </x:c>
       <x:c r="D93" s="6" t="str">
-        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+        <x:v>official_publisher_or_institution_metadata</x:v>
       </x:c>
       <x:c r="E93" s="7" t="d">
         <x:v>2026-10-23T00:00:00.000Z</x:v>
@@ -7704,31 +11393,721 @@
     </x:row>
     <x:row r="94" ht="64" customHeight="1">
       <x:c r="A94" s="6" t="str">
+        <x:v>梁令</x:v>
+      </x:c>
+      <x:c r="B94" s="6" t="str">
+        <x:v>liangling-source-1</x:v>
+      </x:c>
+      <x:c r="C94" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
+      </x:c>
+      <x:c r="D94" s="6" t="str">
+        <x:v>official_roster_read</x:v>
+      </x:c>
+      <x:c r="E94" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F94" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G94" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="64" customHeight="1">
+      <x:c r="A95" s="6" t="str">
+        <x:v>梁令</x:v>
+      </x:c>
+      <x:c r="B95" s="6" t="str">
+        <x:v>liangling-source-2</x:v>
+      </x:c>
+      <x:c r="C95" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/ll/index.htm</x:v>
+      </x:c>
+      <x:c r="D95" s="6" t="str">
+        <x:v>official_publisher_or_institution_metadata</x:v>
+      </x:c>
+      <x:c r="E95" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F95" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G95" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="64" customHeight="1">
+      <x:c r="A96" s="6" t="str">
+        <x:v>梁令</x:v>
+      </x:c>
+      <x:c r="B96" s="6" t="str">
+        <x:v>liangling-source-3</x:v>
+      </x:c>
+      <x:c r="C96" s="6" t="str">
+        <x:v>https://escholarship.org/content/qt6tz615j1/qt6tz615j1.pdf</x:v>
+      </x:c>
+      <x:c r="D96" s="6" t="str">
+        <x:v>official_search_index_only</x:v>
+      </x:c>
+      <x:c r="E96" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F96" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G96" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="64" customHeight="1">
+      <x:c r="A97" s="6" t="str">
+        <x:v>任黎明</x:v>
+      </x:c>
+      <x:c r="B97" s="6" t="str">
+        <x:v>renliming-source-1</x:v>
+      </x:c>
+      <x:c r="C97" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
+      </x:c>
+      <x:c r="D97" s="6" t="str">
+        <x:v>official_roster_read</x:v>
+      </x:c>
+      <x:c r="E97" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F97" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G97" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="64" customHeight="1">
+      <x:c r="A98" s="6" t="str">
+        <x:v>任黎明</x:v>
+      </x:c>
+      <x:c r="B98" s="6" t="str">
+        <x:v>renliming-source-2</x:v>
+      </x:c>
+      <x:c r="C98" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/rlm/index.htm</x:v>
+      </x:c>
+      <x:c r="D98" s="6" t="str">
+        <x:v>official_publisher_or_institution_metadata</x:v>
+      </x:c>
+      <x:c r="E98" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F98" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G98" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="64" customHeight="1">
+      <x:c r="A99" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B99" s="6" t="str">
+        <x:v>sunzhong-source-1</x:v>
+      </x:c>
+      <x:c r="C99" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
+      </x:c>
+      <x:c r="D99" s="6" t="str">
+        <x:v>official_roster_read</x:v>
+      </x:c>
+      <x:c r="E99" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F99" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G99" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="64" customHeight="1">
+      <x:c r="A100" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B100" s="6" t="str">
+        <x:v>sunzhong-source-2</x:v>
+      </x:c>
+      <x:c r="C100" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sz/index.htm</x:v>
+      </x:c>
+      <x:c r="D100" s="6" t="str">
+        <x:v>official_publisher_or_institution_metadata</x:v>
+      </x:c>
+      <x:c r="E100" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F100" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G100" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="64" customHeight="1">
+      <x:c r="A101" s="6" t="str">
+        <x:v>孙雷</x:v>
+      </x:c>
+      <x:c r="B101" s="6" t="str">
+        <x:v>sunlei-source-1</x:v>
+      </x:c>
+      <x:c r="C101" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
+      </x:c>
+      <x:c r="D101" s="6" t="str">
+        <x:v>official_roster_read</x:v>
+      </x:c>
+      <x:c r="E101" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F101" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G101" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="64" customHeight="1">
+      <x:c r="A102" s="6" t="str">
+        <x:v>孙雷</x:v>
+      </x:c>
+      <x:c r="B102" s="6" t="str">
+        <x:v>sunlei-source-2</x:v>
+      </x:c>
+      <x:c r="C102" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/sl/index.htm</x:v>
+      </x:c>
+      <x:c r="D102" s="6" t="str">
+        <x:v>official_public_body_read</x:v>
+      </x:c>
+      <x:c r="E102" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F102" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G102" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="64" customHeight="1">
+      <x:c r="A103" s="6" t="str">
+        <x:v>唐克超</x:v>
+      </x:c>
+      <x:c r="B103" s="6" t="str">
+        <x:v>tangkechao-source-1</x:v>
+      </x:c>
+      <x:c r="C103" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
+      </x:c>
+      <x:c r="D103" s="6" t="str">
+        <x:v>official_roster_read</x:v>
+      </x:c>
+      <x:c r="E103" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F103" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G103" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="64" customHeight="1">
+      <x:c r="A104" s="6" t="str">
+        <x:v>唐克超</x:v>
+      </x:c>
+      <x:c r="B104" s="6" t="str">
+        <x:v>tangkechao-source-2</x:v>
+      </x:c>
+      <x:c r="C104" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/tkc/index.htm</x:v>
+      </x:c>
+      <x:c r="D104" s="6" t="str">
+        <x:v>official_public_body_read</x:v>
+      </x:c>
+      <x:c r="E104" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F104" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G104" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="64" customHeight="1">
+      <x:c r="A105" s="6" t="str">
+        <x:v>唐克超</x:v>
+      </x:c>
+      <x:c r="B105" s="6" t="str">
+        <x:v>tangkechao-source-3</x:v>
+      </x:c>
+      <x:c r="C105" s="6" t="str">
+        <x:v>https://wu.mse.berkeley.edu/publications/Qiu-ChemRev2022.pdf</x:v>
+      </x:c>
+      <x:c r="D105" s="6" t="str">
+        <x:v>official_university_hosted_publisher_pdf_read</x:v>
+      </x:c>
+      <x:c r="E105" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F105" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G105" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="64" customHeight="1">
+      <x:c r="A106" s="6" t="str">
+        <x:v>唐克超</x:v>
+      </x:c>
+      <x:c r="B106" s="6" t="str">
+        <x:v>tangkechao-source-4</x:v>
+      </x:c>
+      <x:c r="C106" s="6" t="str">
+        <x:v>https://news.pku.edu.cn/xwzh/62582c06ccf9436791a074749ee84156.htm</x:v>
+      </x:c>
+      <x:c r="D106" s="6" t="str">
+        <x:v>official_search_index_explicit_mentor_statement_only</x:v>
+      </x:c>
+      <x:c r="E106" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F106" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G106" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="64" customHeight="1">
+      <x:c r="A107" s="6" t="str">
+        <x:v>唐克超</x:v>
+      </x:c>
+      <x:c r="B107" s="6" t="str">
+        <x:v>tangkechao-source-5</x:v>
+      </x:c>
+      <x:c r="C107" s="6" t="str">
+        <x:v>https://profiles.stanford.edu/paul-mcintyre</x:v>
+      </x:c>
+      <x:c r="D107" s="6" t="str">
+        <x:v>official_public_body_read</x:v>
+      </x:c>
+      <x:c r="E107" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F107" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G107" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="64" customHeight="1">
+      <x:c r="A108" s="6" t="str">
+        <x:v>王宗巍</x:v>
+      </x:c>
+      <x:c r="B108" s="6" t="str">
+        <x:v>wangzongwei-source-1</x:v>
+      </x:c>
+      <x:c r="C108" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
+      </x:c>
+      <x:c r="D108" s="6" t="str">
+        <x:v>official_roster_read</x:v>
+      </x:c>
+      <x:c r="E108" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F108" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G108" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="64" customHeight="1">
+      <x:c r="A109" s="6" t="str">
+        <x:v>王宗巍</x:v>
+      </x:c>
+      <x:c r="B109" s="6" t="str">
+        <x:v>wangzongwei-source-2</x:v>
+      </x:c>
+      <x:c r="C109" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wzw/index.htm</x:v>
+      </x:c>
+      <x:c r="D109" s="6" t="str">
+        <x:v>official_public_body_read</x:v>
+      </x:c>
+      <x:c r="E109" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F109" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G109" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="64" customHeight="1">
+      <x:c r="A110" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B110" s="6" t="str">
+        <x:v>wangjinyan-source-1</x:v>
+      </x:c>
+      <x:c r="C110" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
+      </x:c>
+      <x:c r="D110" s="6" t="str">
+        <x:v>official_roster_read</x:v>
+      </x:c>
+      <x:c r="E110" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F110" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G110" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="64" customHeight="1">
+      <x:c r="A111" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B111" s="6" t="str">
+        <x:v>wangjinyan-source-2</x:v>
+      </x:c>
+      <x:c r="C111" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wjy/index.htm</x:v>
+      </x:c>
+      <x:c r="D111" s="6" t="str">
+        <x:v>official_public_body_read</x:v>
+      </x:c>
+      <x:c r="E111" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F111" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G111" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="64" customHeight="1">
+      <x:c r="A112" s="6" t="str">
+        <x:v>王金延</x:v>
+      </x:c>
+      <x:c r="B112" s="6" t="str">
+        <x:v>wangjinyan-source-3</x:v>
+      </x:c>
+      <x:c r="C112" s="6" t="str">
+        <x:v>https://eecs.pku.edu.cn/__local/F/4D/7B/2B226B1469BD496DFDBC63A8F04_CD671777_10B68E.pdf?e=.pdf</x:v>
+      </x:c>
+      <x:c r="D112" s="6" t="str">
+        <x:v>official_university_booklet_pdf_read</x:v>
+      </x:c>
+      <x:c r="E112" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F112" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G112" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="64" customHeight="1">
+      <x:c r="A113" s="6" t="str">
+        <x:v>王茂俊</x:v>
+      </x:c>
+      <x:c r="B113" s="6" t="str">
+        <x:v>wangmaojun-source-1</x:v>
+      </x:c>
+      <x:c r="C113" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/index.htm</x:v>
+      </x:c>
+      <x:c r="D113" s="6" t="str">
+        <x:v>official_roster_read</x:v>
+      </x:c>
+      <x:c r="E113" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F113" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G113" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="64" customHeight="1">
+      <x:c r="A114" s="6" t="str">
+        <x:v>王茂俊</x:v>
+      </x:c>
+      <x:c r="B114" s="6" t="str">
+        <x:v>wangmaojun-source-2</x:v>
+      </x:c>
+      <x:c r="C114" s="6" t="str">
+        <x:v>https://ic.pku.edu.cn/szdw/zzjs/jcwndzx1/wmj/index.htm</x:v>
+      </x:c>
+      <x:c r="D114" s="6" t="str">
+        <x:v>official_public_body_read</x:v>
+      </x:c>
+      <x:c r="E114" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F114" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G114" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="64" customHeight="1">
+      <x:c r="A115" s="6" t="str">
+        <x:v>蔡一茂</x:v>
+      </x:c>
+      <x:c r="B115" s="6" t="str">
+        <x:v>institution-classification-8</x:v>
+      </x:c>
+      <x:c r="C115" s="6" t="str">
+        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+      </x:c>
+      <x:c r="D115" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E115" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F115" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G115" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="64" customHeight="1">
+      <x:c r="A116" s="6" t="str">
+        <x:v>程哲</x:v>
+      </x:c>
+      <x:c r="B116" s="6" t="str">
+        <x:v>institution-classification-14</x:v>
+      </x:c>
+      <x:c r="C116" s="6" t="str">
+        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+      </x:c>
+      <x:c r="D116" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E116" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F116" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G116" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="64" customHeight="1">
+      <x:c r="A117" s="6" t="str">
+        <x:v>傅云义</x:v>
+      </x:c>
+      <x:c r="B117" s="6" t="str">
+        <x:v>institution-classification-6</x:v>
+      </x:c>
+      <x:c r="C117" s="6" t="str">
+        <x:v>https://www.csust.edu.cn/fzgh/info/1016/1662.htm</x:v>
+      </x:c>
+      <x:c r="D117" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E117" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F117" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G117" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="64" customHeight="1">
+      <x:c r="A118" s="6" t="str">
+        <x:v>贺明</x:v>
+      </x:c>
+      <x:c r="B118" s="6" t="str">
+        <x:v>institution-classification-8</x:v>
+      </x:c>
+      <x:c r="C118" s="6" t="str">
+        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+      </x:c>
+      <x:c r="D118" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E118" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F118" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G118" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="64" customHeight="1">
+      <x:c r="A119" s="6" t="str">
         <x:v>贾润东</x:v>
       </x:c>
-      <x:c r="B94" s="6" t="str">
+      <x:c r="B119" s="6" t="str">
         <x:v>institution-classification-6</x:v>
       </x:c>
-      <x:c r="C94" s="6" t="str">
+      <x:c r="C119" s="6" t="str">
         <x:v>https://www.uestc.edu.cn/xxgk/xxls.htm</x:v>
       </x:c>
-      <x:c r="D94" s="6" t="str">
+      <x:c r="D119" s="6" t="str">
         <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
       </x:c>
-      <x:c r="E94" s="7" t="d">
-        <x:v>2026-10-23T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="F94" s="6" t="str">
-        <x:v>pku</x:v>
-      </x:c>
-      <x:c r="G94" s="6" t="str">
+      <x:c r="E119" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F119" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G119" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="64" customHeight="1">
+      <x:c r="A120" s="6" t="str">
+        <x:v>黎明</x:v>
+      </x:c>
+      <x:c r="B120" s="6" t="str">
+        <x:v>institution-classification-2</x:v>
+      </x:c>
+      <x:c r="C120" s="6" t="str">
+        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+      </x:c>
+      <x:c r="D120" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E120" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F120" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G120" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="64" customHeight="1">
+      <x:c r="A121" s="6" t="str">
+        <x:v>任黎明</x:v>
+      </x:c>
+      <x:c r="B121" s="6" t="str">
+        <x:v>institution-classification-2</x:v>
+      </x:c>
+      <x:c r="C121" s="6" t="str">
+        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+      </x:c>
+      <x:c r="D121" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E121" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F121" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G121" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="64" customHeight="1">
+      <x:c r="A122" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B122" s="6" t="str">
+        <x:v>institution-classification-2</x:v>
+      </x:c>
+      <x:c r="C122" s="6" t="str">
+        <x:v>https://www.csust.edu.cn/fzgh/info/1016/1662.htm</x:v>
+      </x:c>
+      <x:c r="D122" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E122" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F122" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G122" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="64" customHeight="1">
+      <x:c r="A123" s="6" t="str">
+        <x:v>孙仲</x:v>
+      </x:c>
+      <x:c r="B123" s="6" t="str">
+        <x:v>institution-classification-3</x:v>
+      </x:c>
+      <x:c r="C123" s="6" t="str">
+        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+      </x:c>
+      <x:c r="D123" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E123" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F123" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G123" s="6" t="str">
+        <x:v>北京大学</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="64" customHeight="1">
+      <x:c r="A124" s="6" t="str">
+        <x:v>王茂俊</x:v>
+      </x:c>
+      <x:c r="B124" s="6" t="str">
+        <x:v>institution-classification-2</x:v>
+      </x:c>
+      <x:c r="C124" s="6" t="str">
+        <x:v>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</x:v>
+      </x:c>
+      <x:c r="D124" s="6" t="str">
+        <x:v>历史985院校分类参考；非个人授位或就读当年建设身份的证明</x:v>
+      </x:c>
+      <x:c r="E124" s="7" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="F124" s="6" t="str">
+        <x:v>pku</x:v>
+      </x:c>
+      <x:c r="G124" s="6" t="str">
         <x:v>北京大学</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d29f4c6c3e0406d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d32c4db4b704620"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>